<commit_message>
feat: consolidate skill vfx effects
</commit_message>
<xml_diff>
--- a/Project 2048/Docs/Project2048_Balancing_Template.xlsx
+++ b/Project 2048/Docs/Project2048_Balancing_Template.xlsx
@@ -1523,7 +1523,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B12" s="62" t="inlineStr">
         <is>
-          <t>SkillSO 42개 / EnemySO 12개 / PrototypePlayer.asset / CostConverter.cs / RewardTableSO</t>
+          <t>SkillSO 41개 / EnemySO 12개 / PrototypePlayer.asset / CostConverter.cs / RewardTableSO</t>
         </is>
       </c>
       <c r="C12" s="51" t="n"/>
@@ -2193,7 +2193,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3150,7 +3150,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3572,20 +3572,20 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart ns1:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3614,7 +3614,7 @@
     <row r="2" ht="19.5" customHeight="1">
       <c r="A2" s="73" t="inlineStr">
         <is>
-          <t>SkillSO 42 assets synced from Assets/Data/Skills</t>
+          <t>SkillSO 41 assets synced from Assets/Data/Skills</t>
         </is>
       </c>
       <c r="I2" s="51" t="n"/>
@@ -3753,7 +3753,7 @@
         <v>40</v>
       </c>
       <c r="J5" s="74">
-        <f>IF(OR($C5&lt;&gt;"Attack",$I5&lt;=0),0,CEILING(($I5/10)*(IF($E5="ShieldHp",Inputs!$B$34,IF($E5="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C5&lt;&gt;"Attack",$I5&lt;=0),0,CEILING(($I5/10)*(IF($E5="ShieldHp",Inputs!$B$33,IF($E5="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K5" s="75" t="n">
@@ -3777,12 +3777,12 @@
     <row r="6">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>feint-strike</t>
+          <t>overburn</t>
         </is>
       </c>
       <c r="B6" s="45" t="inlineStr">
         <is>
-          <t>방어 읽기</t>
+          <t>초과연소</t>
         </is>
       </c>
       <c r="C6" s="45" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="D6" s="70" t="inlineStr">
         <is>
-          <t>FeintStrike</t>
+          <t>OverburnAttack</t>
         </is>
       </c>
       <c r="E6" s="70" t="inlineStr">
@@ -3809,13 +3809,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="63" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I6" s="63" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="J6" s="74">
-        <f>IF(OR($C6&lt;&gt;"Attack",$I6&lt;=0),0,CEILING(($I6/10)*(IF($E6="ShieldHp",Inputs!$B$34,IF($E6="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C6&lt;&gt;"Attack",$I6&lt;=0),0,CEILING(($I6/10)*(IF($E6="ShieldHp",Inputs!$B$33,IF($E6="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K6" s="75" t="n">
@@ -3827,24 +3827,24 @@
       </c>
       <c r="M6" s="77" t="inlineStr">
         <is>
-          <t>적에게 위력 40 피해를 준다. 대상이 직전 턴에 방어 또는 회복 유형 스킬을 사용했다면 위력 80으로 공격하고 보호막의 50%를 관통한다.</t>
+          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다.</t>
         </is>
       </c>
       <c r="N6" s="78" t="inlineStr">
         <is>
-          <t>적에게 위력 40 피해를 준다. 대상이 직전 턴에 방어 또는 회복 유형 스킬을 사용했다면 위력 80으로 공격하고 보호막의 50%를 관통한다.</t>
+          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>overburn</t>
+          <t>poison-coat</t>
         </is>
       </c>
       <c r="B7" s="45" t="inlineStr">
         <is>
-          <t>초과연소</t>
+          <t>독 묻히기</t>
         </is>
       </c>
       <c r="C7" s="45" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="D7" s="70" t="inlineStr">
         <is>
-          <t>OverburnAttack</t>
+          <t>PoisonAttack</t>
         </is>
       </c>
       <c r="E7" s="70" t="inlineStr">
@@ -3871,13 +3871,13 @@
         <v>5</v>
       </c>
       <c r="H7" s="63" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="I7" s="63" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J7" s="74">
-        <f>IF(OR($C7&lt;&gt;"Attack",$I7&lt;=0),0,CEILING(($I7/10)*(IF($E7="ShieldHp",Inputs!$B$34,IF($E7="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C7&lt;&gt;"Attack",$I7&lt;=0),0,CEILING(($I7/10)*(IF($E7="ShieldHp",Inputs!$B$33,IF($E7="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K7" s="75" t="n">
@@ -3889,24 +3889,24 @@
       </c>
       <c r="M7" s="77" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다.</t>
+          <t>적에게 위력 30 피해를 주고 독 3턴을 부여한다. 독은 대상 턴 종료 시 최대 체력의 5% 피해를 주며 최소 1 피해를 준다.</t>
         </is>
       </c>
       <c r="N7" s="78" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다.</t>
+          <t>적에게 위력 30 피해를 주고 독 3턴을 부여한다. 독은 대상 턴 종료 시 최대 체력의 5% 피해를 주며 최소 1 피해를 준다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>poison-coat</t>
+          <t>shield-bash</t>
         </is>
       </c>
       <c r="B8" s="45" t="inlineStr">
         <is>
-          <t>독 묻히기</t>
+          <t>방패 밀치기</t>
         </is>
       </c>
       <c r="C8" s="45" t="inlineStr">
@@ -3916,12 +3916,12 @@
       </c>
       <c r="D8" s="70" t="inlineStr">
         <is>
-          <t>PoisonAttack</t>
+          <t>ShieldScalingAttack</t>
         </is>
       </c>
       <c r="E8" s="70" t="inlineStr">
         <is>
-          <t>AttackPower</t>
+          <t>ShieldHp</t>
         </is>
       </c>
       <c r="F8" s="70" t="inlineStr">
@@ -3933,13 +3933,13 @@
         <v>5</v>
       </c>
       <c r="H8" s="63" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="I8" s="63" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J8" s="74">
-        <f>IF(OR($C8&lt;&gt;"Attack",$I8&lt;=0),0,CEILING(($I8/10)*(IF($E8="ShieldHp",Inputs!$B$34,IF($E8="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C8&lt;&gt;"Attack",$I8&lt;=0),0,CEILING(($I8/10)*(IF($E8="ShieldHp",Inputs!$B$33,IF($E8="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K8" s="75" t="n">
@@ -3951,24 +3951,24 @@
       </c>
       <c r="M8" s="77" t="inlineStr">
         <is>
-          <t>적에게 위력 30 피해를 주고 독 3턴을 부여한다. 독은 대상 턴 종료 시 최대 체력의 5% 피해를 주며 최소 1 피해를 준다.</t>
+          <t>현재 보호막 수치로 계산하여 적에게 위력 60 피해를 준다. 보호막은 소모하지 않는다.</t>
         </is>
       </c>
       <c r="N8" s="78" t="inlineStr">
         <is>
-          <t>적에게 위력 30 피해를 주고 독 3턴을 부여한다. 독은 대상 턴 종료 시 최대 체력의 5% 피해를 주며 최소 1 피해를 준다.</t>
+          <t>현재 보호막 수치로 계산하여 적에게 위력 60 피해를 준다. 보호막은 소모하지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>shield-bash</t>
+          <t>bleeding-cut</t>
         </is>
       </c>
       <c r="B9" s="45" t="inlineStr">
         <is>
-          <t>방패 밀치기</t>
+          <t>화염구</t>
         </is>
       </c>
       <c r="C9" s="45" t="inlineStr">
@@ -3978,12 +3978,12 @@
       </c>
       <c r="D9" s="70" t="inlineStr">
         <is>
-          <t>ShieldScalingAttack</t>
+          <t>OverburnAttack</t>
         </is>
       </c>
       <c r="E9" s="70" t="inlineStr">
         <is>
-          <t>ShieldHp</t>
+          <t>AttackPower</t>
         </is>
       </c>
       <c r="F9" s="70" t="inlineStr">
@@ -3992,16 +3992,16 @@
         </is>
       </c>
       <c r="G9" s="70" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H9" s="63" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I9" s="63" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J9" s="74">
-        <f>IF(OR($C9&lt;&gt;"Attack",$I9&lt;=0),0,CEILING(($I9/10)*(IF($E9="ShieldHp",Inputs!$B$34,IF($E9="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C9&lt;&gt;"Attack",$I9&lt;=0),0,CEILING(($I9/10)*(IF($E9="ShieldHp",Inputs!$B$33,IF($E9="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K9" s="75" t="n">
@@ -4013,86 +4013,86 @@
       </c>
       <c r="M9" s="77" t="inlineStr">
         <is>
-          <t>현재 보호막 수치로 계산하여 적에게 위력 60 피해를 준다. 보호막은 소모하지 않는다.</t>
+          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 화염구를 발사한다.</t>
         </is>
       </c>
       <c r="N9" s="78" t="inlineStr">
         <is>
-          <t>현재 보호막 수치로 계산하여 적에게 위력 60 피해를 준다. 보호막은 소모하지 않는다.</t>
+          <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 화염구를 발사한다.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="45" t="inlineStr">
-        <is>
-          <t>bleeding-cut</t>
-        </is>
-      </c>
-      <c r="B10" s="45" t="inlineStr">
-        <is>
-          <t>출혈 베기</t>
-        </is>
-      </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>execute</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>마무리</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>BleedAttack</t>
-        </is>
-      </c>
-      <c r="E10" s="70" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ExecuteAttack</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>AttackPower</t>
         </is>
       </c>
-      <c r="F10" s="70" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Shared</t>
         </is>
       </c>
-      <c r="G10" s="70" t="n">
+      <c r="G10" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="63" t="n">
-        <v>50</v>
-      </c>
-      <c r="I10" s="63" t="n">
-        <v>50</v>
-      </c>
-      <c r="J10" s="74">
-        <f>IF(OR($C10&lt;&gt;"Attack",$I10&lt;=0),0,CEILING(($I10/10)*(IF($E10="ShieldHp",Inputs!$B$34,IF($E10="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
-        <v/>
-      </c>
-      <c r="K10" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="76">
+      <c r="H10" t="n">
+        <v>40</v>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" s="79">
+        <f>IF(OR($C10&lt;&gt;"Attack",$I10&lt;=0),0,CEILING(($I10/10)*(IF($E10="ShieldHp",Inputs!$B$33,IF($E10="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
+        <v/>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="79">
         <f>IF($G10=0,"",$J10/$G10)</f>
         <v/>
       </c>
-      <c r="M10" s="77" t="inlineStr">
-        <is>
-          <t>적에게 위력 50 피해를 주고 출혈 2턴을 부여한다. 출혈 상태인 대상은 공격을 받을 때마다 추가 피해 20을 받는다.</t>
-        </is>
-      </c>
-      <c r="N10" s="78" t="inlineStr">
-        <is>
-          <t>적에게 위력 50 피해를 주고 출혈 2턴을 부여한다. 출혈 상태인 대상은 공격을 받을 때마다 추가 피해 20을 받는다.</t>
+      <c r="M10" s="79" t="inlineStr">
+        <is>
+          <t>적에게 위력 40 피해를 준다. 대상의 현재 체력이 최대 체력의 30% 이하라면 위력 80으로 공격한다.</t>
+        </is>
+      </c>
+      <c r="N10" s="79" t="inlineStr">
+        <is>
+          <t>적에게 위력 40 피해를 준다. 대상의 현재 체력이 최대 체력의 30% 이하라면 위력 80으로 공격한다.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>execute</t>
+          <t>gather-light</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>마무리</t>
+          <t>빛 모으기</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ExecuteAttack</t>
+          <t>ChargeAttack</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4112,20 +4112,20 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>6</v>
       </c>
       <c r="H11" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="J11" s="79">
-        <f>IF(OR($C11&lt;&gt;"Attack",$I11&lt;=0),0,CEILING(($I11/10)*(IF($E11="ShieldHp",Inputs!$B$34,IF($E11="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C11&lt;&gt;"Attack",$I11&lt;=0),0,CEILING(($I11/10)*(IF($E11="ShieldHp",Inputs!$B$33,IF($E11="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K11" t="n">
@@ -4137,24 +4137,24 @@
       </c>
       <c r="M11" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 40 피해를 준다. 대상의 현재 체력이 최대 체력의 30% 이하라면 위력 80으로 공격한다.</t>
+          <t>이번 턴에는 빛을 모은다. 다음 플레이어 턴 시작 시 적에게 위력 120의 빛 공격을 자동으로 사용한다.</t>
         </is>
       </c>
       <c r="N11" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 40 피해를 준다. 대상의 현재 체력이 최대 체력의 30% 이하라면 위력 80으로 공격한다.</t>
+          <t>이번 턴에는 빛을 모은다. 다음 플레이어 턴 시작 시 적에게 위력 120의 빛 공격을 자동으로 사용한다.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gather-light</t>
+          <t>light-shot</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>빛 모으기</t>
+          <t>빛 발사</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ChargeAttack</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4181,13 +4181,13 @@
         <v>6</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J12" s="79">
-        <f>IF(OR($C12&lt;&gt;"Attack",$I12&lt;=0),0,CEILING(($I12/10)*(IF($E12="ShieldHp",Inputs!$B$34,IF($E12="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C12&lt;&gt;"Attack",$I12&lt;=0),0,CEILING(($I12/10)*(IF($E12="ShieldHp",Inputs!$B$33,IF($E12="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K12" t="n">
@@ -4199,24 +4199,24 @@
       </c>
       <c r="M12" s="79" t="inlineStr">
         <is>
-          <t>이번 턴에는 빛을 모은다. 다음 플레이어 턴 시작 시 적에게 위력 120의 빛 공격을 자동으로 사용한다.</t>
+          <t>적에게 위력 60의 빛 피해를 준다.</t>
         </is>
       </c>
       <c r="N12" s="79" t="inlineStr">
         <is>
-          <t>이번 턴에는 빛을 모은다. 다음 플레이어 턴 시작 시 적에게 위력 120의 빛 공격을 자동으로 사용한다.</t>
+          <t>적에게 위력 60의 빛 피해를 준다.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>light-shot</t>
+          <t>tentacle-strike</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>빛 발사</t>
+          <t>촉수 치기</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4224,9 +4224,9 @@
           <t>Attack</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>BasicAttack</t>
+      <c r="D13" s="79" t="inlineStr">
+        <is>
+          <t>BoardMovePenaltyAttack</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4236,20 +4236,20 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>6</v>
       </c>
       <c r="H13" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="I13" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J13" s="79">
-        <f>IF(OR($C13&lt;&gt;"Attack",$I13&lt;=0),0,CEILING(($I13/10)*(IF($E13="ShieldHp",Inputs!$B$34,IF($E13="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C13&lt;&gt;"Attack",$I13&lt;=0),0,CEILING(($I13/10)*(IF($E13="ShieldHp",Inputs!$B$33,IF($E13="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K13" t="n">
@@ -4261,24 +4261,24 @@
       </c>
       <c r="M13" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 60의 빛 피해를 준다.</t>
+          <t>적에게 위력 90 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 감소한다.</t>
         </is>
       </c>
       <c r="N13" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 60의 빛 피해를 준다.</t>
+          <t>적에게 위력 90 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 감소한다.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tentacle-strike</t>
+          <t>blood-fang</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>촉수 치기</t>
+          <t>불사르기</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4286,9 +4286,9 @@
           <t>Attack</t>
         </is>
       </c>
-      <c r="D14" s="79" t="inlineStr">
-        <is>
-          <t>BoardMovePenaltyAttack</t>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SacrificeAttack</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4302,16 +4302,16 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H14" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="I14" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J14" s="79">
-        <f>IF(OR($C14&lt;&gt;"Attack",$I14&lt;=0),0,CEILING(($I14/10)*(IF($E14="ShieldHp",Inputs!$B$34,IF($E14="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C14&lt;&gt;"Attack",$I14&lt;=0),0,CEILING(($I14/10)*(IF($E14="ShieldHp",Inputs!$B$33,IF($E14="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K14" t="n">
@@ -4323,24 +4323,24 @@
       </c>
       <c r="M14" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 90 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 감소한다.</t>
+          <t>최대 체력의 10%를 불태워 화염구를 발사하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
       <c r="N14" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 90 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 감소한다.</t>
+          <t>최대 체력의 10%를 불태워 화염구를 발사하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>blood-fang</t>
+          <t>body-press</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>피의 이빨</t>
+          <t>육중한 압박</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4350,12 +4350,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SacrificeAttack</t>
+          <t>DefenseScalingAttack</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AttackPower</t>
+          <t>DefensePower</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -4367,13 +4367,13 @@
         <v>7</v>
       </c>
       <c r="H15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="J15" s="79">
-        <f>IF(OR($C15&lt;&gt;"Attack",$I15&lt;=0),0,CEILING(($I15/10)*(IF($E15="ShieldHp",Inputs!$B$34,IF($E15="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C15&lt;&gt;"Attack",$I15&lt;=0),0,CEILING(($I15/10)*(IF($E15="ShieldHp",Inputs!$B$33,IF($E15="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K15" t="n">
@@ -4385,24 +4385,24 @@
       </c>
       <c r="M15" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 10%를 지불하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
+          <t>공격력 대신 방어력으로 계산하여 적에게 위력 80 피해를 준다.</t>
         </is>
       </c>
       <c r="N15" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 10%를 지불하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
+          <t>공격력 대신 방어력으로 계산하여 적에게 위력 80 피해를 준다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>body-press</t>
+          <t>flow-strike</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>육중한 압박</t>
+          <t>흐름 가르기</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4412,30 +4412,30 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DefenseScalingAttack</t>
+          <t>BoardMoveBonusAttack</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DefensePower</t>
+          <t>AttackPower</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>7</v>
       </c>
       <c r="H16" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="I16" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="J16" s="79">
-        <f>IF(OR($C16&lt;&gt;"Attack",$I16&lt;=0),0,CEILING(($I16/10)*(IF($E16="ShieldHp",Inputs!$B$34,IF($E16="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C16&lt;&gt;"Attack",$I16&lt;=0),0,CEILING(($I16/10)*(IF($E16="ShieldHp",Inputs!$B$33,IF($E16="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K16" t="n">
@@ -4447,24 +4447,24 @@
       </c>
       <c r="M16" s="79" t="inlineStr">
         <is>
-          <t>공격력 대신 방어력으로 계산하여 적에게 위력 80 피해를 준다.</t>
+          <t>적에게 위력 50 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 증가한다.</t>
         </is>
       </c>
       <c r="N16" s="79" t="inlineStr">
         <is>
-          <t>공격력 대신 방어력으로 계산하여 적에게 위력 80 피해를 준다.</t>
+          <t>적에게 위력 50 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 증가한다.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>flow-strike</t>
+          <t>intimidating-shot</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>흐름 가르기</t>
+          <t>위협 사격</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BoardMoveBonusAttack</t>
+          <t>AttackStageDown</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -4497,7 +4497,7 @@
         <v>50</v>
       </c>
       <c r="J17" s="79">
-        <f>IF(OR($C17&lt;&gt;"Attack",$I17&lt;=0),0,CEILING(($I17/10)*(IF($E17="ShieldHp",Inputs!$B$34,IF($E17="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C17&lt;&gt;"Attack",$I17&lt;=0),0,CEILING(($I17/10)*(IF($E17="ShieldHp",Inputs!$B$33,IF($E17="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K17" t="n">
@@ -4509,24 +4509,24 @@
       </c>
       <c r="M17" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 증가한다.</t>
+          <t>적에게 위력 50 피해를 주고, 적의 공격 랭크를 1 낮춘다. [Rank multiplier: enemy attack -1 =&gt; attack x0.67]</t>
         </is>
       </c>
       <c r="N17" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 증가한다.</t>
+          <t>적에게 위력 50 피해를 주고, 적의 공격 랭크를 1 낮춘다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>intimidating-shot</t>
+          <t>life-drain</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>위협 사격</t>
+          <t>생명 흡수</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AttackStageDown</t>
+          <t>LifeStealAttack</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4553,13 +4553,13 @@
         <v>7</v>
       </c>
       <c r="H18" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I18" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J18" s="79">
-        <f>IF(OR($C18&lt;&gt;"Attack",$I18&lt;=0),0,CEILING(($I18/10)*(IF($E18="ShieldHp",Inputs!$B$34,IF($E18="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C18&lt;&gt;"Attack",$I18&lt;=0),0,CEILING(($I18/10)*(IF($E18="ShieldHp",Inputs!$B$33,IF($E18="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K18" t="n">
@@ -4571,24 +4571,24 @@
       </c>
       <c r="M18" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 주고, 적의 공격 랭크를 1 낮춘다. [Rank multiplier: enemy attack -1 =&gt; attack x0.67]</t>
+          <t>적에게 위력 60 피해를 준다. 실제 체력 피해의 50%만큼 체력을 회복한다.</t>
         </is>
       </c>
       <c r="N18" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 50 피해를 주고, 적의 공격 랭크를 1 낮춘다.</t>
+          <t>적에게 위력 60 피해를 준다. 실제 체력 피해의 50%만큼 체력을 회복한다.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>life-drain</t>
+          <t>open-wound</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>생명 흡수</t>
+          <t>폭렬</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LifeStealAttack</t>
+          <t>OverburnAttack</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4615,13 +4615,15 @@
         <v>7</v>
       </c>
       <c r="H19" t="n">
-        <v>60</v>
-      </c>
-      <c r="I19" t="n">
-        <v>60</v>
+        <v>70</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="J19" s="79">
-        <f>IF(OR($C19&lt;&gt;"Attack",$I19&lt;=0),0,CEILING(($I19/10)*(IF($E19="ShieldHp",Inputs!$B$34,IF($E19="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C19&lt;&gt;"Attack",$I19&lt;=0),0,CEILING(($I19/10)*(IF($E19="ShieldHp",Inputs!$B$33,IF($E19="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K19" t="n">
@@ -4633,24 +4635,24 @@
       </c>
       <c r="M19" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 60 피해를 준다. 실제 체력 피해의 50%만큼 체력을 회복한다.</t>
+          <t>적에게 위력 70 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 폭발하는 화염구를 발사하고, 적중 시 적 위치에 폭발 이펙트를 일으킨다.</t>
         </is>
       </c>
       <c r="N19" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 60 피해를 준다. 실제 체력 피해의 50%만큼 체력을 회복한다.</t>
+          <t>적에게 위력 70 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 폭발하는 화염구를 발사하고, 적중 시 적 위치에 폭발 이펙트를 일으킨다.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>open-wound</t>
+          <t>shield-burst</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>상처 벌리기</t>
+          <t>방패 폭발</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4660,12 +4662,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OpenWoundAttack</t>
+          <t>ShieldBurstAttack</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AttackPower</t>
+          <t>ShieldHp</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4677,13 +4679,13 @@
         <v>7</v>
       </c>
       <c r="H20" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="I20" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="J20" s="79">
-        <f>IF(OR($C20&lt;&gt;"Attack",$I20&lt;=0),0,CEILING(($I20/10)*(IF($E20="ShieldHp",Inputs!$B$34,IF($E20="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C20&lt;&gt;"Attack",$I20&lt;=0),0,CEILING(($I20/10)*(IF($E20="ShieldHp",Inputs!$B$33,IF($E20="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K20" t="n">
@@ -4695,24 +4697,24 @@
       </c>
       <c r="M20" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 70 피해를 준다. 대상이 독 또는 출혈 상태라면 위력 120으로 공격하고 해당 상태들의 지속시간을 1턴 늘린다.</t>
+          <t>현재 보호막 수치로 계산하여 적에게 위력 100 피해를 준다. 사용 후 보호막을 모두 잃는다.</t>
         </is>
       </c>
       <c r="N20" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 70 피해를 준다. 대상이 독 또는 출혈 상태라면 위력 120으로 공격하고 해당 상태들의 지속시간을 1턴 늘린다.</t>
+          <t>현재 보호막 수치로 계산하여 적에게 위력 100 피해를 준다. 사용 후 보호막을 모두 잃는다.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>shield-burst</t>
+          <t>bioluminescence</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>방패 폭발</t>
+          <t>생체 발광</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4722,30 +4724,30 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ShieldBurstAttack</t>
+          <t>SacrificeAttack</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ShieldHp</t>
+          <t>AttackPower</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H21" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="I21" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="J21" s="79">
-        <f>IF(OR($C21&lt;&gt;"Attack",$I21&lt;=0),0,CEILING(($I21/10)*(IF($E21="ShieldHp",Inputs!$B$34,IF($E21="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C21&lt;&gt;"Attack",$I21&lt;=0),0,CEILING(($I21/10)*(IF($E21="ShieldHp",Inputs!$B$33,IF($E21="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K21" t="n">
@@ -4757,24 +4759,24 @@
       </c>
       <c r="M21" s="79" t="inlineStr">
         <is>
-          <t>현재 보호막 수치로 계산하여 적에게 위력 100 피해를 준다. 사용 후 보호막을 모두 잃는다.</t>
+          <t>최대 체력의 25%를 지불하고 적에게 위력 120 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
       <c r="N21" s="79" t="inlineStr">
         <is>
-          <t>현재 보호막 수치로 계산하여 적에게 위력 100 피해를 준다. 사용 후 보호막을 모두 잃는다.</t>
+          <t>최대 체력의 25%를 지불하고 적에게 위력 120 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>bioluminescence</t>
+          <t>heavy-strike</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>생체 발광</t>
+          <t>강타</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4784,7 +4786,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SacrificeAttack</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4794,20 +4796,20 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>8</v>
       </c>
       <c r="H22" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="I22" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="J22" s="79">
-        <f>IF(OR($C22&lt;&gt;"Attack",$I22&lt;=0),0,CEILING(($I22/10)*(IF($E22="ShieldHp",Inputs!$B$34,IF($E22="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C22&lt;&gt;"Attack",$I22&lt;=0),0,CEILING(($I22/10)*(IF($E22="ShieldHp",Inputs!$B$33,IF($E22="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K22" t="n">
@@ -4819,24 +4821,24 @@
       </c>
       <c r="M22" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 25%를 지불하고 적에게 위력 120 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
+          <t>적에게 위력 80 피해를 준다.</t>
         </is>
       </c>
       <c r="N22" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 25%를 지불하고 적에게 위력 120 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
+          <t>적에게 위력 80 피해를 준다.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>heavy-strike</t>
+          <t>reckless-blow</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>강타</t>
+          <t>무리한 강타</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4844,9 +4846,9 @@
           <t>Attack</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>BasicAttack</t>
+      <c r="D23" s="79" t="inlineStr">
+        <is>
+          <t>BoardMovePenaltyAttack</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4863,13 +4865,13 @@
         <v>8</v>
       </c>
       <c r="H23" t="n">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="I23" t="n">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="J23" s="79">
-        <f>IF(OR($C23&lt;&gt;"Attack",$I23&lt;=0),0,CEILING(($I23/10)*(IF($E23="ShieldHp",Inputs!$B$34,IF($E23="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C23&lt;&gt;"Attack",$I23&lt;=0),0,CEILING(($I23/10)*(IF($E23="ShieldHp",Inputs!$B$33,IF($E23="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K23" t="n">
@@ -4881,34 +4883,34 @@
       </c>
       <c r="M23" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 80 피해를 준다.</t>
+          <t>적에게 위력 110 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
         </is>
       </c>
       <c r="N23" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 80 피해를 준다.</t>
+          <t>적에게 위력 110 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>reckless-blow</t>
+          <t>crack-brand</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>무리한 강타</t>
+          <t>균열 낙인</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="D24" s="79" t="inlineStr">
-        <is>
-          <t>BoardMovePenaltyAttack</t>
+          <t>Debuff</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CrackBrand</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4922,16 +4924,16 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H24" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="J24" s="79">
-        <f>IF(OR($C24&lt;&gt;"Attack",$I24&lt;=0),0,CEILING(($I24/10)*(IF($E24="ShieldHp",Inputs!$B$34,IF($E24="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C24&lt;&gt;"Attack",$I24&lt;=0),0,CEILING(($I24/10)*(IF($E24="ShieldHp",Inputs!$B$33,IF($E24="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K24" t="n">
@@ -4943,24 +4945,24 @@
       </c>
       <c r="M24" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 110 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
+          <t>대상에게 낙인을 부여한다. 낙인이 있는 대상이 다음 공격을 받으면 추가 피해 40을 받고 낙인이 해제된다.</t>
         </is>
       </c>
       <c r="N24" s="79" t="inlineStr">
         <is>
-          <t>적에게 위력 110 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
+          <t>대상에게 낙인을 부여한다. 낙인이 있는 대상이 다음 공격을 받으면 추가 피해 40을 받고 낙인이 해제된다.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>crack-brand</t>
+          <t>flash</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>균열 낙인</t>
+          <t>섬광</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4970,7 +4972,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CrackBrand</t>
+          <t>AttackStageDown</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4993,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="J25" s="79">
-        <f>IF(OR($C25&lt;&gt;"Attack",$I25&lt;=0),0,CEILING(($I25/10)*(IF($E25="ShieldHp",Inputs!$B$34,IF($E25="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C25&lt;&gt;"Attack",$I25&lt;=0),0,CEILING(($I25/10)*(IF($E25="ShieldHp",Inputs!$B$33,IF($E25="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K25" t="n">
@@ -5005,24 +5007,24 @@
       </c>
       <c r="M25" s="79" t="inlineStr">
         <is>
-          <t>대상에게 낙인을 부여한다. 낙인이 있는 대상이 다음 공격을 받으면 추가 피해 40을 받고 낙인이 해제된다.</t>
+          <t>적의 공격 랭크를 1 낮춘다. [Rank multiplier: enemy attack -1 =&gt; attack x0.67]</t>
         </is>
       </c>
       <c r="N25" s="79" t="inlineStr">
         <is>
-          <t>대상에게 낙인을 부여한다. 낙인이 있는 대상이 다음 공격을 받으면 추가 피해 40을 받고 낙인이 해제된다.</t>
+          <t>적의 공격 랭크를 1 낮춘다.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>flash</t>
+          <t>howl</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>섬광</t>
+          <t>울부짖기</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5032,7 +5034,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AttackStageDown</t>
+          <t>DefenseStageDown</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5055,7 +5057,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="79">
-        <f>IF(OR($C26&lt;&gt;"Attack",$I26&lt;=0),0,CEILING(($I26/10)*(IF($E26="ShieldHp",Inputs!$B$34,IF($E26="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C26&lt;&gt;"Attack",$I26&lt;=0),0,CEILING(($I26/10)*(IF($E26="ShieldHp",Inputs!$B$33,IF($E26="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K26" t="n">
@@ -5067,24 +5069,24 @@
       </c>
       <c r="M26" s="79" t="inlineStr">
         <is>
-          <t>적의 공격 랭크를 1 낮춘다. [Rank multiplier: enemy attack -1 =&gt; attack x0.67]</t>
+          <t>적의 방어 랭크를 1 낮춘다. [Rank multiplier: enemy defense -1 =&gt; defense x0.67]</t>
         </is>
       </c>
       <c r="N26" s="79" t="inlineStr">
         <is>
-          <t>적의 공격 랭크를 1 낮춘다.</t>
+          <t>적의 방어 랭크를 1 낮춘다.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>howl</t>
+          <t>taunt</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>울부짖기</t>
+          <t>도발</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5094,7 +5096,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>DefenseStageDown</t>
+          <t>Taunt</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5104,7 +5106,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -5117,7 +5119,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="79">
-        <f>IF(OR($C27&lt;&gt;"Attack",$I27&lt;=0),0,CEILING(($I27/10)*(IF($E27="ShieldHp",Inputs!$B$34,IF($E27="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C27&lt;&gt;"Attack",$I27&lt;=0),0,CEILING(($I27/10)*(IF($E27="ShieldHp",Inputs!$B$33,IF($E27="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K27" t="n">
@@ -5129,24 +5131,24 @@
       </c>
       <c r="M27" s="79" t="inlineStr">
         <is>
-          <t>적의 방어 랭크를 1 낮춘다. [Rank multiplier: enemy defense -1 =&gt; defense x0.67]</t>
+          <t>적의 다음 행동 인텐드를 공격으로 강제하고, 적의 공격 랭크를 2 올린다. [Rank multiplier: enemy attack +2 =&gt; attack x2]</t>
         </is>
       </c>
       <c r="N27" s="79" t="inlineStr">
         <is>
-          <t>적의 방어 랭크를 1 낮춘다.</t>
+          <t>적의 다음 행동 인텐드를 공격으로 강제하고, 적의 공격 랭크를 2 올린다.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>taunt</t>
+          <t>seal-skill</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>도발</t>
+          <t>봉인</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5156,7 +5158,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Taunt</t>
+          <t>SealSkill</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5166,11 +5168,11 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -5179,7 +5181,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="79">
-        <f>IF(OR($C28&lt;&gt;"Attack",$I28&lt;=0),0,CEILING(($I28/10)*(IF($E28="ShieldHp",Inputs!$B$34,IF($E28="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C28&lt;&gt;"Attack",$I28&lt;=0),0,CEILING(($I28/10)*(IF($E28="ShieldHp",Inputs!$B$33,IF($E28="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K28" t="n">
@@ -5191,34 +5193,34 @@
       </c>
       <c r="M28" s="79" t="inlineStr">
         <is>
-          <t>적의 다음 행동 인텐드를 공격으로 강제하고, 적의 공격 랭크를 2 올린다. [Rank multiplier: enemy attack +2 =&gt; attack x2]</t>
+          <t>대상이 마지막으로 사용한 비기본 스킬을 다음 턴 1회 사용할 수 없게 한다. 봉인할 스킬이 없으면 효과가 없다.</t>
         </is>
       </c>
       <c r="N28" s="79" t="inlineStr">
         <is>
-          <t>적의 다음 행동 인텐드를 공격으로 강제하고, 적의 공격 랭크를 2 올린다.</t>
+          <t>대상이 마지막으로 사용한 비기본 스킬을 다음 턴 1회 사용할 수 없게 한다. 봉인할 스킬이 없으면 효과가 없다.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>seal-skill</t>
+          <t>afterglow-save</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>봉인</t>
+          <t>잔광 저장</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Debuff</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SealSkill</t>
+          <t>CostCarry</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5228,11 +5230,11 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -5241,7 +5243,7 @@
         <v>0</v>
       </c>
       <c r="J29" s="79">
-        <f>IF(OR($C29&lt;&gt;"Attack",$I29&lt;=0),0,CEILING(($I29/10)*(IF($E29="ShieldHp",Inputs!$B$34,IF($E29="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C29&lt;&gt;"Attack",$I29&lt;=0),0,CEILING(($I29/10)*(IF($E29="ShieldHp",Inputs!$B$33,IF($E29="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K29" t="n">
@@ -5253,24 +5255,24 @@
       </c>
       <c r="M29" s="79" t="inlineStr">
         <is>
-          <t>대상이 마지막으로 사용한 비기본 스킬을 다음 턴 1회 사용할 수 없게 한다. 봉인할 스킬이 없으면 효과가 없다.</t>
+          <t>이번 턴 종료 시 남은 코스트를 최대 4까지 다음 턴으로 이월한다. 이월 코스트는 한 번 적용되면 사라진다.</t>
         </is>
       </c>
       <c r="N29" s="79" t="inlineStr">
         <is>
-          <t>대상이 마지막으로 사용한 비기본 스킬을 다음 턴 1회 사용할 수 없게 한다. 봉인할 스킬이 없으면 효과가 없다.</t>
+          <t>이번 턴 종료 시 남은 코스트를 최대 4까지 다음 턴으로 이월한다. 이월 코스트는 한 번 적용되면 사라진다.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>afterglow-save</t>
+          <t>cleanse-hand</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>잔광 저장</t>
+          <t>정화의 손길</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5280,7 +5282,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CostCarry</t>
+          <t>DarknessCleanse</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5303,7 +5305,7 @@
         <v>0</v>
       </c>
       <c r="J30" s="79">
-        <f>IF(OR($C30&lt;&gt;"Attack",$I30&lt;=0),0,CEILING(($I30/10)*(IF($E30="ShieldHp",Inputs!$B$34,IF($E30="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C30&lt;&gt;"Attack",$I30&lt;=0),0,CEILING(($I30/10)*(IF($E30="ShieldHp",Inputs!$B$33,IF($E30="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K30" t="n">
@@ -5315,24 +5317,24 @@
       </c>
       <c r="M30" s="79" t="inlineStr">
         <is>
-          <t>이번 턴 종료 시 남은 코스트를 최대 4까지 다음 턴으로 이월한다. 이월 코스트는 한 번 적용되면 사라진다.</t>
+          <t>보드 위 암흑 장애물 1개를 제거한다. 제거에 성공하면 코스트 2를 환급한다.</t>
         </is>
       </c>
       <c r="N30" s="79" t="inlineStr">
         <is>
-          <t>이번 턴 종료 시 남은 코스트를 최대 4까지 다음 턴으로 이월한다. 이월 코스트는 한 번 적용되면 사라진다.</t>
+          <t>보드 위 암흑 장애물 1개를 제거한다. 제거에 성공하면 코스트 2를 환급한다.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cleanse-hand</t>
+          <t>focus-breath</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>정화의 손길</t>
+          <t>집중 호흡</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5342,7 +5344,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DarknessCleanse</t>
+          <t>CriticalStageUp</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5352,7 +5354,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -5365,7 +5367,7 @@
         <v>0</v>
       </c>
       <c r="J31" s="79">
-        <f>IF(OR($C31&lt;&gt;"Attack",$I31&lt;=0),0,CEILING(($I31/10)*(IF($E31="ShieldHp",Inputs!$B$34,IF($E31="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C31&lt;&gt;"Attack",$I31&lt;=0),0,CEILING(($I31/10)*(IF($E31="ShieldHp",Inputs!$B$33,IF($E31="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K31" t="n">
@@ -5377,24 +5379,24 @@
       </c>
       <c r="M31" s="79" t="inlineStr">
         <is>
-          <t>보드 위 암흑 장애물 1개를 제거한다. 제거에 성공하면 코스트 2를 환급한다.</t>
+          <t>치명타 랭크를 1 올린다. [Critical rank: +1 =&gt; critical chance +20%p]</t>
         </is>
       </c>
       <c r="N31" s="79" t="inlineStr">
         <is>
-          <t>보드 위 암흑 장애물 1개를 제거한다. 제거에 성공하면 코스트 2를 환급한다.</t>
+          <t>치명타 랭크를 1 올린다.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>focus-breath</t>
+          <t>low-stance</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>집중 호흡</t>
+          <t>낮은 자세</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5404,7 +5406,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CriticalStageUp</t>
+          <t>BasicDefense</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5421,17 +5423,17 @@
         <v>4</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J32" s="79">
-        <f>IF(OR($C32&lt;&gt;"Attack",$I32&lt;=0),0,CEILING(($I32/10)*(IF($E32="ShieldHp",Inputs!$B$34,IF($E32="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C32&lt;&gt;"Attack",$I32&lt;=0),0,CEILING(($I32/10)*(IF($E32="ShieldHp",Inputs!$B$33,IF($E32="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L32" s="79">
         <f>IF($G32=0,"",$J32/$G32)</f>
@@ -5439,24 +5441,24 @@
       </c>
       <c r="M32" s="79" t="inlineStr">
         <is>
-          <t>치명타 랭크를 1 올린다. [Critical rank: +1 =&gt; critical chance +20%p]</t>
+          <t>보호막 30을 얻는다.</t>
         </is>
       </c>
       <c r="N32" s="79" t="inlineStr">
         <is>
-          <t>치명타 랭크를 1 올린다.</t>
+          <t>보호막 30을 얻는다.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>low-stance</t>
+          <t>light-echo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>낮은 자세</t>
+          <t>빛의 메아리</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5464,9 +5466,9 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>BasicDefense</t>
+      <c r="D33" s="79" t="inlineStr">
+        <is>
+          <t>NextAttackPowerMultiplier</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5476,24 +5478,24 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H33" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="J33" s="79">
-        <f>IF(OR($C33&lt;&gt;"Attack",$I33&lt;=0),0,CEILING(($I33/10)*(IF($E33="ShieldHp",Inputs!$B$34,IF($E33="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C33&lt;&gt;"Attack",$I33&lt;=0),0,CEILING(($I33/10)*(IF($E33="ShieldHp",Inputs!$B$33,IF($E33="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K33" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L33" s="79">
         <f>IF($G33=0,"",$J33/$G33)</f>
@@ -5501,24 +5503,24 @@
       </c>
       <c r="M33" s="79" t="inlineStr">
         <is>
-          <t>보호막 30을 얻는다.</t>
+          <t>다음 공격의 기술 위력이 1.3배가 된다.</t>
         </is>
       </c>
       <c r="N33" s="79" t="inlineStr">
         <is>
-          <t>보호막 30을 얻는다.</t>
+          <t>다음 공격의 기술 위력이 1.3배가 된다.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>light-echo</t>
+          <t>endure</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>빛의 메아리</t>
+          <t>이악물기</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5526,9 +5528,9 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="D34" s="79" t="inlineStr">
-        <is>
-          <t>NextAttackPowerMultiplier</t>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Endure</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5538,11 +5540,11 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -5551,7 +5553,7 @@
         <v>0</v>
       </c>
       <c r="J34" s="79">
-        <f>IF(OR($C34&lt;&gt;"Attack",$I34&lt;=0),0,CEILING(($I34/10)*(IF($E34="ShieldHp",Inputs!$B$34,IF($E34="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C34&lt;&gt;"Attack",$I34&lt;=0),0,CEILING(($I34/10)*(IF($E34="ShieldHp",Inputs!$B$33,IF($E34="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K34" t="n">
@@ -5563,24 +5565,24 @@
       </c>
       <c r="M34" s="79" t="inlineStr">
         <is>
-          <t>다음 공격의 기술 위력이 1.3배가 된다.</t>
+          <t>다음 적 턴 동안 체력이 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
       <c r="N34" s="79" t="inlineStr">
         <is>
-          <t>다음 공격의 기술 위력이 1.3배가 된다.</t>
+          <t>다음 적 턴 동안 체력이 1 아래로 내려가지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>endure</t>
+          <t>iron-wall</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>이악물기</t>
+          <t>철벽</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5590,7 +5592,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Endure</t>
+          <t>DefenseStageUp</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5613,7 +5615,7 @@
         <v>0</v>
       </c>
       <c r="J35" s="79">
-        <f>IF(OR($C35&lt;&gt;"Attack",$I35&lt;=0),0,CEILING(($I35/10)*(IF($E35="ShieldHp",Inputs!$B$34,IF($E35="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C35&lt;&gt;"Attack",$I35&lt;=0),0,CEILING(($I35/10)*(IF($E35="ShieldHp",Inputs!$B$33,IF($E35="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K35" t="n">
@@ -5625,24 +5627,24 @@
       </c>
       <c r="M35" s="79" t="inlineStr">
         <is>
-          <t>다음 적 턴 동안 체력이 1 아래로 내려가지 않는다.</t>
+          <t>내 방어 랭크를 2 올린다. [Rank multiplier: self defense +2 =&gt; defense x2]</t>
         </is>
       </c>
       <c r="N35" s="79" t="inlineStr">
         <is>
-          <t>다음 적 턴 동안 체력이 1 아래로 내려가지 않는다.</t>
+          <t>내 방어 랭크를 2 올린다.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>iron-wall</t>
+          <t>light-guard</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>철벽</t>
+          <t>빛 방어</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5652,7 +5654,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>DefenseStageUp</t>
+          <t>BasicDefense</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5662,24 +5664,24 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G36" t="n">
         <v>6</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J36" s="79">
-        <f>IF(OR($C36&lt;&gt;"Attack",$I36&lt;=0),0,CEILING(($I36/10)*(IF($E36="ShieldHp",Inputs!$B$34,IF($E36="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C36&lt;&gt;"Attack",$I36&lt;=0),0,CEILING(($I36/10)*(IF($E36="ShieldHp",Inputs!$B$33,IF($E36="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L36" s="79">
         <f>IF($G36=0,"",$J36/$G36)</f>
@@ -5687,24 +5689,24 @@
       </c>
       <c r="M36" s="79" t="inlineStr">
         <is>
-          <t>내 방어 랭크를 2 올린다. [Rank multiplier: self defense +2 =&gt; defense x2]</t>
+          <t>보호막 60을 얻는다.</t>
         </is>
       </c>
       <c r="N36" s="79" t="inlineStr">
         <is>
-          <t>내 방어 랭크를 2 올린다.</t>
+          <t>보호막 60을 얻는다.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>light-guard</t>
+          <t>light-split</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>빛 방어</t>
+          <t>빛의 분산</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5714,7 +5716,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>BasicDefense</t>
+          <t>NextAttackSplit</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5731,17 +5733,17 @@
         <v>6</v>
       </c>
       <c r="H37" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="J37" s="79">
-        <f>IF(OR($C37&lt;&gt;"Attack",$I37&lt;=0),0,CEILING(($I37/10)*(IF($E37="ShieldHp",Inputs!$B$34,IF($E37="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C37&lt;&gt;"Attack",$I37&lt;=0),0,CEILING(($I37/10)*(IF($E37="ShieldHp",Inputs!$B$33,IF($E37="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K37" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="L37" s="79">
         <f>IF($G37=0,"",$J37/$G37)</f>
@@ -5749,24 +5751,24 @@
       </c>
       <c r="M37" s="79" t="inlineStr">
         <is>
-          <t>보호막 60을 얻는다.</t>
+          <t>다음 공격이 2회 공격으로 바뀐다. 각 공격은 원래 기술 위력의 60%로 계산된다.</t>
         </is>
       </c>
       <c r="N37" s="79" t="inlineStr">
         <is>
-          <t>보호막 60을 얻는다.</t>
+          <t>다음 공격이 2회 공격으로 바뀐다. 각 공격은 원래 기술 위력의 60%로 계산된다.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>light-split</t>
+          <t>sharp-senses</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>빛의 분산</t>
+          <t>예리한 감각</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5776,7 +5778,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>NextAttackSplit</t>
+          <t>CriticalStageUp</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5786,7 +5788,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -5799,7 +5801,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="79">
-        <f>IF(OR($C38&lt;&gt;"Attack",$I38&lt;=0),0,CEILING(($I38/10)*(IF($E38="ShieldHp",Inputs!$B$34,IF($E38="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C38&lt;&gt;"Attack",$I38&lt;=0),0,CEILING(($I38/10)*(IF($E38="ShieldHp",Inputs!$B$33,IF($E38="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K38" t="n">
@@ -5811,24 +5813,24 @@
       </c>
       <c r="M38" s="79" t="inlineStr">
         <is>
-          <t>다음 공격이 2회 공격으로 바뀐다. 각 공격은 원래 기술 위력의 60%로 계산된다.</t>
+          <t>치명타 랭크를 2 올린다. [Critical rank: +2 =&gt; critical chance +40%p]</t>
         </is>
       </c>
       <c r="N38" s="79" t="inlineStr">
         <is>
-          <t>다음 공격이 2회 공격으로 바뀐다. 각 공격은 원래 기술 위력의 60%로 계산된다.</t>
+          <t>치명타 랭크를 2 올린다.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>sharp-senses</t>
+          <t>thorn-guard</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>예리한 감각</t>
+          <t>가시 방어</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5838,7 +5840,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CriticalStageUp</t>
+          <t>ThornGuard</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5852,20 +5854,20 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J39" s="79">
-        <f>IF(OR($C39&lt;&gt;"Attack",$I39&lt;=0),0,CEILING(($I39/10)*(IF($E39="ShieldHp",Inputs!$B$34,IF($E39="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C39&lt;&gt;"Attack",$I39&lt;=0),0,CEILING(($I39/10)*(IF($E39="ShieldHp",Inputs!$B$33,IF($E39="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L39" s="79">
         <f>IF($G39=0,"",$J39/$G39)</f>
@@ -5873,34 +5875,34 @@
       </c>
       <c r="M39" s="79" t="inlineStr">
         <is>
-          <t>치명타 랭크를 2 올린다. [Critical rank: +2 =&gt; critical chance +40%p]</t>
+          <t>보호막 40을 얻는다. 보호막이 남아 있을 때 적의 직접 공격을 받으면, 현재 보호막 수치로 위력 40 반격을 한다.</t>
         </is>
       </c>
       <c r="N39" s="79" t="inlineStr">
         <is>
-          <t>치명타 랭크를 2 올린다.</t>
+          <t>보호막 40을 얻는다. 보호막이 남아 있을 때 적의 직접 공격을 받으면, 현재 보호막 수치로 위력 40 반격을 한다.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>thorn-guard</t>
+          <t>light-recover</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>가시 방어</t>
+          <t>빛 회복</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Heal</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ThornGuard</t>
+          <t>Heal</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -5910,24 +5912,24 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>PlayerOnly</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H40" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J40" s="79">
-        <f>IF(OR($C40&lt;&gt;"Attack",$I40&lt;=0),0,CEILING(($I40/10)*(IF($E40="ShieldHp",Inputs!$B$34,IF($E40="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C40&lt;&gt;"Attack",$I40&lt;=0),0,CEILING(($I40/10)*(IF($E40="ShieldHp",Inputs!$B$33,IF($E40="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K40" t="n">
-        <v>40</v>
+        <v>0.25</v>
       </c>
       <c r="L40" s="79">
         <f>IF($G40=0,"",$J40/$G40)</f>
@@ -5935,34 +5937,34 @@
       </c>
       <c r="M40" s="79" t="inlineStr">
         <is>
-          <t>보호막 40을 얻는다. 보호막이 남아 있을 때 적의 직접 공격을 받으면, 현재 보호막 수치로 위력 40 반격을 한다.</t>
+          <t>최대 체력의 25%만큼 회복한다.</t>
         </is>
       </c>
       <c r="N40" s="79" t="inlineStr">
         <is>
-          <t>보호막 40을 얻는다. 보호막이 남아 있을 때 적의 직접 공격을 받으면, 현재 보호막 수치로 위력 40 반격을 한다.</t>
+          <t>최대 체력의 25%만큼 회복한다.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>light-recover</t>
+          <t>dark-shackle</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>빛 회복</t>
+          <t>어둠의 족쇄</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Heal</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Heal</t>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="D41" s="79" t="inlineStr">
+        <is>
+          <t>BoardMovePenaltyAttack</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5972,24 +5974,24 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PlayerOnly</t>
+          <t>EnemyOnly</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J41" s="79">
-        <f>IF(OR($C41&lt;&gt;"Attack",$I41&lt;=0),0,CEILING(($I41/10)*(IF($E41="ShieldHp",Inputs!$B$34,IF($E41="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C41&lt;&gt;"Attack",$I41&lt;=0),0,CEILING(($I41/10)*(IF($E41="ShieldHp",Inputs!$B$33,IF($E41="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K41" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="L41" s="79">
         <f>IF($G41=0,"",$J41/$G41)</f>
@@ -5997,34 +5999,34 @@
       </c>
       <c r="M41" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 25%만큼 회복한다.</t>
+          <t>위력 40 피해를 주고, 다음 플레이어 턴의 보드 이동 횟수를 1 줄인다.</t>
         </is>
       </c>
       <c r="N41" s="79" t="inlineStr">
         <is>
-          <t>최대 체력의 25%만큼 회복한다.</t>
+          <t>위력 40 피해를 주고, 다음 플레이어 턴의 보드 이동 횟수를 1 줄인다.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>dark-shackle</t>
+          <t>black-corrosion</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>어둠의 족쇄</t>
+          <t>검은 부식</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="D42" s="79" t="inlineStr">
-        <is>
-          <t>BoardMovePenaltyAttack</t>
+          <t>Debuff</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CostGainDown</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -6041,13 +6043,13 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J42" s="79">
-        <f>IF(OR($C42&lt;&gt;"Attack",$I42&lt;=0),0,CEILING(($I42/10)*(IF($E42="ShieldHp",Inputs!$B$34,IF($E42="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C42&lt;&gt;"Attack",$I42&lt;=0),0,CEILING(($I42/10)*(IF($E42="ShieldHp",Inputs!$B$33,IF($E42="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K42" t="n">
@@ -6059,24 +6061,24 @@
       </c>
       <c r="M42" s="79" t="inlineStr">
         <is>
-          <t>위력 40 피해를 주고, 다음 플레이어 턴의 보드 이동 횟수를 1 줄인다.</t>
+          <t>플레이어의 다음 턴 코스트 획득량에서 3을 차감한다. 코스트 획득량은 0 미만으로 내려가지 않는다.</t>
         </is>
       </c>
       <c r="N42" s="79" t="inlineStr">
         <is>
-          <t>위력 40 피해를 주고, 다음 플레이어 턴의 보드 이동 횟수를 1 줄인다.</t>
+          <t>플레이어의 다음 턴 코스트 획득량에서 3을 차감한다. 코스트 획득량은 0 미만으로 내려가지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>black-corrosion</t>
+          <t>black-pressure</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>검은 부식</t>
+          <t>검은 압박</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6109,7 +6111,7 @@
         <v>0</v>
       </c>
       <c r="J43" s="79">
-        <f>IF(OR($C43&lt;&gt;"Attack",$I43&lt;=0),0,CEILING(($I43/10)*(IF($E43="ShieldHp",Inputs!$B$34,IF($E43="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C43&lt;&gt;"Attack",$I43&lt;=0),0,CEILING(($I43/10)*(IF($E43="ShieldHp",Inputs!$B$33,IF($E43="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K43" t="n">
@@ -6121,24 +6123,24 @@
       </c>
       <c r="M43" s="79" t="inlineStr">
         <is>
-          <t>플레이어의 다음 턴 코스트 획득량에서 3을 차감한다. 코스트 획득량은 0 미만으로 내려가지 않는다.</t>
+          <t>다음 플레이어 턴에 보드에서 얻는 코스트가 30% 감소한다.</t>
         </is>
       </c>
       <c r="N43" s="79" t="inlineStr">
         <is>
-          <t>플레이어의 다음 턴 코스트 획득량에서 3을 차감한다. 코스트 획득량은 0 미만으로 내려가지 않는다.</t>
+          <t>다음 플레이어 턴에 보드에서 얻는 코스트가 30% 감소한다.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>black-pressure</t>
+          <t>darkness</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>검은 압박</t>
+          <t>암흑</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6148,7 +6150,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CostGainDown</t>
+          <t>BoardObstacleDebuff</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6171,7 +6173,7 @@
         <v>0</v>
       </c>
       <c r="J44" s="79">
-        <f>IF(OR($C44&lt;&gt;"Attack",$I44&lt;=0),0,CEILING(($I44/10)*(IF($E44="ShieldHp",Inputs!$B$34,IF($E44="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C44&lt;&gt;"Attack",$I44&lt;=0),0,CEILING(($I44/10)*(IF($E44="ShieldHp",Inputs!$B$33,IF($E44="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K44" t="n">
@@ -6183,24 +6185,24 @@
       </c>
       <c r="M44" s="79" t="inlineStr">
         <is>
-          <t>다음 플레이어 턴에 보드에서 얻는 코스트가 30% 감소한다.</t>
+          <t>다음 플레이어 보드에 암흑 장애물 1개를 생성한다.</t>
         </is>
       </c>
       <c r="N44" s="79" t="inlineStr">
         <is>
-          <t>다음 플레이어 턴에 보드에서 얻는 코스트가 30% 감소한다.</t>
+          <t>다음 플레이어 보드에 암흑 장애물 1개를 생성한다.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>darkness</t>
+          <t>deep-darkness</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>암흑</t>
+          <t>깊은 암흑</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6233,7 +6235,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="79">
-        <f>IF(OR($C45&lt;&gt;"Attack",$I45&lt;=0),0,CEILING(($I45/10)*(IF($E45="ShieldHp",Inputs!$B$34,IF($E45="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
+        <f>IF(OR($C45&lt;&gt;"Attack",$I45&lt;=0),0,CEILING(($I45/10)*(IF($E45="ShieldHp",Inputs!$B$33,IF($E45="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v/>
       </c>
       <c r="K45" t="n">
@@ -6245,79 +6247,17 @@
       </c>
       <c r="M45" s="79" t="inlineStr">
         <is>
-          <t>다음 플레이어 보드에 암흑 장애물 1개를 생성한다.</t>
+          <t>다음 플레이어 보드에 암흑 장애물 2개를 생성한다.</t>
         </is>
       </c>
       <c r="N45" s="79" t="inlineStr">
         <is>
-          <t>다음 플레이어 보드에 암흑 장애물 1개를 생성한다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>deep-darkness</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>깊은 암흑</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Debuff</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>BoardObstacleDebuff</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>AttackPower</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>EnemyOnly</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" s="79">
-        <f>IF(OR($C46&lt;&gt;"Attack",$I46&lt;=0),0,CEILING(($I46/10)*(IF($E46="ShieldHp",Inputs!$B$34,IF($E46="DefensePower",Inputs!$B$29,Inputs!$B$5))/MAX(1,Inputs!$B$33))*Inputs!$B$35,1))</f>
-        <v/>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" s="79">
-        <f>IF($G46=0,"",$J46/$G46)</f>
-        <v/>
-      </c>
-      <c r="M46" s="79" t="inlineStr">
-        <is>
           <t>다음 플레이어 보드에 암흑 장애물 2개를 생성한다.</t>
         </is>
       </c>
-      <c r="N46" s="79" t="inlineStr">
-        <is>
-          <t>다음 플레이어 보드에 암흑 장애물 2개를 생성한다.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K5:L10">
+  <conditionalFormatting sqref="K5:L9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6330,22 +6270,22 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="C5:C46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$H$2:$H$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -7934,13 +7874,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -9516,18 +9456,18 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10428,7 +10368,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>상처 벌리기</t>
+          <t>폭렬</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -10465,7 +10405,7 @@
       </c>
       <c r="Q18" s="79" t="inlineStr">
         <is>
-          <t>상처 벌리기 기술을 배웁니다.</t>
+          <t>폭렬 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
@@ -10531,7 +10471,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>learn-feint-strike</t>
+          <t>learn-overburn</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -10546,7 +10486,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>방어 읽기</t>
+          <t>초과연소</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -10583,14 +10523,14 @@
       </c>
       <c r="Q20" s="79" t="inlineStr">
         <is>
-          <t>방어 읽기 기술을 배웁니다.</t>
+          <t>초과연소 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>learn-overburn</t>
+          <t>learn-seal-skill</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -10605,7 +10545,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>초과연소</t>
+          <t>봉인</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -10642,14 +10582,14 @@
       </c>
       <c r="Q21" s="79" t="inlineStr">
         <is>
-          <t>초과연소 기술을 배웁니다.</t>
+          <t>봉인 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>learn-seal-skill</t>
+          <t>learn-taunt</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -10664,7 +10604,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>봉인</t>
+          <t>도발</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -10701,14 +10641,14 @@
       </c>
       <c r="Q22" s="79" t="inlineStr">
         <is>
-          <t>봉인 기술을 배웁니다.</t>
+          <t>도발 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>learn-taunt</t>
+          <t>learn-crack-brand</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -10723,7 +10663,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>도발</t>
+          <t>균열 낙인</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -10760,14 +10700,14 @@
       </c>
       <c r="Q23" s="79" t="inlineStr">
         <is>
-          <t>도발 기술을 배웁니다.</t>
+          <t>균열 낙인 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>learn-crack-brand</t>
+          <t>learn-afterglow-save</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10782,7 +10722,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>균열 낙인</t>
+          <t>잔광 저장</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -10819,14 +10759,14 @@
       </c>
       <c r="Q24" s="79" t="inlineStr">
         <is>
-          <t>균열 낙인 기술을 배웁니다.</t>
+          <t>잔광 저장 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>learn-afterglow-save</t>
+          <t>learn-cleanse-hand</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -10841,7 +10781,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>잔광 저장</t>
+          <t>정화의 손길</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -10878,68 +10818,14 @@
       </c>
       <c r="Q25" s="79" t="inlineStr">
         <is>
-          <t>잔광 저장 기술을 배웁니다.</t>
+          <t>정화의 손길 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>learn-cleanse-hand</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>기술 습득</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>LearnSkill</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>정화의 손길</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F26" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" t="n">
-        <v>1</v>
-      </c>
       <c r="H26" s="79" t="n"/>
       <c r="I26" s="79" t="n"/>
-      <c r="J26" t="n">
-        <v>2</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q26" s="79" t="inlineStr">
-        <is>
-          <t>정화의 손길 기술을 배웁니다.</t>
-        </is>
-      </c>
+      <c r="Q26" s="79" t="n"/>
     </row>
     <row r="27">
       <c r="H27" s="79" t="n"/>
@@ -10947,40 +10833,61 @@
       <c r="Q27" s="79" t="n"/>
     </row>
     <row r="28">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B28" s="67" t="inlineStr">
+        <is>
+          <t>Difficulty</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="inlineStr">
+        <is>
+          <t>Remaining Moves</t>
+        </is>
+      </c>
+      <c r="D28" s="67" t="inlineStr">
+        <is>
+          <t>OverCost</t>
+        </is>
+      </c>
+      <c r="E28" s="67" t="inlineStr">
+        <is>
+          <t>Turn Count</t>
+        </is>
+      </c>
+      <c r="F28" s="67" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
       <c r="H28" s="79" t="n"/>
       <c r="I28" s="79" t="n"/>
       <c r="Q28" s="79" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="67" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B29" s="67" t="inlineStr">
-        <is>
-          <t>Difficulty</t>
-        </is>
-      </c>
-      <c r="C29" s="67" t="inlineStr">
-        <is>
-          <t>Remaining Moves</t>
-        </is>
-      </c>
-      <c r="D29" s="67" t="inlineStr">
-        <is>
-          <t>OverCost</t>
-        </is>
-      </c>
-      <c r="E29" s="67" t="inlineStr">
-        <is>
-          <t>Turn Count</t>
-        </is>
-      </c>
-      <c r="F29" s="67" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>빠른 승리</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="79">
+        <f>MAX(Inputs!$B$16,$B29*Inputs!$B$12+$C29*Inputs!$B$13+$D29*Inputs!$B$14-$E29*Inputs!$B$15)</f>
+        <v/>
       </c>
       <c r="H29" s="79" t="n"/>
       <c r="I29" s="79" t="n"/>
@@ -10989,20 +10896,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>빠른 승리</t>
+          <t>표준 승리</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
         <v>2</v>
       </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F30" s="79">
         <f>MAX(Inputs!$B$16,$B30*Inputs!$B$12+$C30*Inputs!$B$13+$D30*Inputs!$B$14-$E30*Inputs!$B$15)</f>
@@ -11015,20 +10922,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>표준 승리</t>
+          <t>고난도 빠른 승리</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" s="79">
         <f>MAX(Inputs!$B$16,$B31*Inputs!$B$12+$C31*Inputs!$B$13+$D31*Inputs!$B$14-$E31*Inputs!$B$15)</f>
@@ -11041,20 +10948,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>고난도 빠른 승리</t>
+          <t>고난도 장기전</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F32" s="79">
         <f>MAX(Inputs!$B$16,$B32*Inputs!$B$12+$C32*Inputs!$B$13+$D32*Inputs!$B$14-$E32*Inputs!$B$15)</f>
@@ -11064,44 +10971,18 @@
       <c r="I32" s="79" t="n"/>
       <c r="Q32" s="79" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>고난도 장기전</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4</v>
-      </c>
-      <c r="E33" t="n">
-        <v>9</v>
-      </c>
-      <c r="F33" s="79">
-        <f>MAX(Inputs!$B$16,$B33*Inputs!$B$12+$C33*Inputs!$B$13+$D33*Inputs!$B$14-$E33*Inputs!$B$15)</f>
-        <v/>
-      </c>
-      <c r="H33" s="79" t="n"/>
-      <c r="I33" s="79" t="n"/>
-      <c r="Q33" s="79" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
   <tableParts count="2">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart ns1:id="rId2"/>
+    <tablePart ns1:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -11378,7 +11259,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11530,7 +11411,7 @@
       </c>
       <c r="G3" s="45" t="inlineStr">
         <is>
-          <t>방어 읽기</t>
+          <t>초과연소</t>
         </is>
       </c>
       <c r="H3" s="45" t="inlineStr">
@@ -11569,7 +11450,7 @@
       </c>
       <c r="G4" s="45" t="inlineStr">
         <is>
-          <t>초과연소</t>
+          <t>독 묻히기</t>
         </is>
       </c>
       <c r="H4" s="45" t="inlineStr">
@@ -11604,7 +11485,7 @@
       </c>
       <c r="G5" s="45" t="inlineStr">
         <is>
-          <t>독 묻히기</t>
+          <t>방패 밀치기</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -11631,7 +11512,7 @@
       </c>
       <c r="G6" s="45" t="inlineStr">
         <is>
-          <t>방패 밀치기</t>
+          <t>출혈 베기</t>
         </is>
       </c>
       <c r="H6" s="45" t="n"/>
@@ -11654,7 +11535,7 @@
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>출혈 베기</t>
+          <t>마무리</t>
         </is>
       </c>
       <c r="H7" s="45" t="n"/>
@@ -11672,7 +11553,7 @@
       </c>
       <c r="G8" s="45" t="inlineStr">
         <is>
-          <t>마무리</t>
+          <t>빛 모으기</t>
         </is>
       </c>
       <c r="H8" s="45" t="n"/>
@@ -11690,7 +11571,7 @@
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>빛 모으기</t>
+          <t>빛 발사</t>
         </is>
       </c>
       <c r="H9" s="45" t="n"/>
@@ -11708,7 +11589,7 @@
       </c>
       <c r="G10" s="45" t="inlineStr">
         <is>
-          <t>빛 발사</t>
+          <t>촉수 치기</t>
         </is>
       </c>
       <c r="H10" s="45" t="n"/>
@@ -11726,7 +11607,7 @@
       </c>
       <c r="G11" s="45" t="inlineStr">
         <is>
-          <t>촉수 치기</t>
+          <t>피의 이빨</t>
         </is>
       </c>
       <c r="H11" s="45" t="n"/>
@@ -11744,7 +11625,7 @@
       </c>
       <c r="G12" s="45" t="inlineStr">
         <is>
-          <t>피의 이빨</t>
+          <t>육중한 압박</t>
         </is>
       </c>
       <c r="H12" s="45" t="n"/>
@@ -11762,7 +11643,7 @@
       </c>
       <c r="G13" s="45" t="inlineStr">
         <is>
-          <t>육중한 압박</t>
+          <t>흐름 가르기</t>
         </is>
       </c>
       <c r="H13" s="45" t="n"/>
@@ -11776,7 +11657,7 @@
       <c r="F14" s="45" t="n"/>
       <c r="G14" s="45" t="inlineStr">
         <is>
-          <t>흐름 가르기</t>
+          <t>위협 사격</t>
         </is>
       </c>
       <c r="H14" s="45" t="n"/>
@@ -11790,7 +11671,7 @@
       <c r="F15" s="45" t="n"/>
       <c r="G15" s="45" t="inlineStr">
         <is>
-          <t>위협 사격</t>
+          <t>생명 흡수</t>
         </is>
       </c>
       <c r="H15" s="45" t="n"/>
@@ -11804,7 +11685,7 @@
       <c r="F16" s="45" t="n"/>
       <c r="G16" s="45" t="inlineStr">
         <is>
-          <t>생명 흡수</t>
+          <t>상처 벌리기</t>
         </is>
       </c>
       <c r="H16" s="45" t="n"/>
@@ -11818,7 +11699,7 @@
       <c r="F17" s="45" t="n"/>
       <c r="G17" s="45" t="inlineStr">
         <is>
-          <t>상처 벌리기</t>
+          <t>방패 폭발</t>
         </is>
       </c>
       <c r="H17" s="45" t="n"/>
@@ -11832,7 +11713,7 @@
       <c r="F18" s="45" t="n"/>
       <c r="G18" s="45" t="inlineStr">
         <is>
-          <t>방패 폭발</t>
+          <t>생체 발광</t>
         </is>
       </c>
       <c r="H18" s="45" t="n"/>
@@ -11846,7 +11727,7 @@
       <c r="F19" s="45" t="n"/>
       <c r="G19" s="45" t="inlineStr">
         <is>
-          <t>생체 발광</t>
+          <t>강타</t>
         </is>
       </c>
       <c r="H19" s="45" t="n"/>
@@ -11860,7 +11741,7 @@
       <c r="F20" s="45" t="n"/>
       <c r="G20" s="45" t="inlineStr">
         <is>
-          <t>강타</t>
+          <t>무리한 강타</t>
         </is>
       </c>
       <c r="H20" s="45" t="n"/>
@@ -11874,7 +11755,7 @@
       <c r="F21" s="45" t="n"/>
       <c r="G21" s="45" t="inlineStr">
         <is>
-          <t>무리한 강타</t>
+          <t>균열 낙인</t>
         </is>
       </c>
       <c r="H21" s="45" t="n"/>
@@ -11888,7 +11769,7 @@
       <c r="F22" s="45" t="n"/>
       <c r="G22" s="45" t="inlineStr">
         <is>
-          <t>균열 낙인</t>
+          <t>섬광</t>
         </is>
       </c>
       <c r="H22" s="45" t="n"/>
@@ -11902,7 +11783,7 @@
       <c r="F23" s="45" t="n"/>
       <c r="G23" s="45" t="inlineStr">
         <is>
-          <t>섬광</t>
+          <t>울부짖기</t>
         </is>
       </c>
       <c r="H23" s="45" t="n"/>
@@ -11916,7 +11797,7 @@
       <c r="F24" s="45" t="n"/>
       <c r="G24" s="45" t="inlineStr">
         <is>
-          <t>울부짖기</t>
+          <t>도발</t>
         </is>
       </c>
       <c r="H24" s="45" t="n"/>
@@ -11930,7 +11811,7 @@
       <c r="F25" s="45" t="n"/>
       <c r="G25" s="45" t="inlineStr">
         <is>
-          <t>도발</t>
+          <t>봉인</t>
         </is>
       </c>
       <c r="H25" s="45" t="n"/>
@@ -11944,7 +11825,7 @@
       <c r="F26" s="45" t="n"/>
       <c r="G26" s="45" t="inlineStr">
         <is>
-          <t>봉인</t>
+          <t>잔광 저장</t>
         </is>
       </c>
       <c r="H26" s="45" t="n"/>
@@ -11958,7 +11839,7 @@
       <c r="F27" s="45" t="n"/>
       <c r="G27" s="45" t="inlineStr">
         <is>
-          <t>잔광 저장</t>
+          <t>정화의 손길</t>
         </is>
       </c>
       <c r="H27" s="45" t="n"/>
@@ -11972,7 +11853,7 @@
       <c r="F28" s="45" t="n"/>
       <c r="G28" s="45" t="inlineStr">
         <is>
-          <t>정화의 손길</t>
+          <t>집중 호흡</t>
         </is>
       </c>
       <c r="H28" s="45" t="n"/>
@@ -11986,7 +11867,7 @@
       <c r="F29" s="45" t="n"/>
       <c r="G29" s="45" t="inlineStr">
         <is>
-          <t>집중 호흡</t>
+          <t>낮은 자세</t>
         </is>
       </c>
       <c r="H29" s="45" t="n"/>
@@ -12000,7 +11881,7 @@
       <c r="F30" s="45" t="n"/>
       <c r="G30" s="45" t="inlineStr">
         <is>
-          <t>낮은 자세</t>
+          <t>빛의 메아리</t>
         </is>
       </c>
       <c r="H30" s="45" t="n"/>
@@ -12008,91 +11889,91 @@
     <row r="31">
       <c r="G31" t="inlineStr">
         <is>
-          <t>빛의 메아리</t>
+          <t>이악물기</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="G32" t="inlineStr">
         <is>
-          <t>이악물기</t>
+          <t>철벽</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="G33" t="inlineStr">
         <is>
-          <t>철벽</t>
+          <t>빛 방어</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="G34" t="inlineStr">
         <is>
-          <t>빛 방어</t>
+          <t>빛의 분산</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="G35" t="inlineStr">
         <is>
-          <t>빛의 분산</t>
+          <t>예리한 감각</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="G36" t="inlineStr">
         <is>
-          <t>예리한 감각</t>
+          <t>가시 방어</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="G37" t="inlineStr">
         <is>
-          <t>가시 방어</t>
+          <t>빛 회복</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="G38" t="inlineStr">
         <is>
-          <t>빛 회복</t>
+          <t>어둠의 족쇄</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="G39" t="inlineStr">
         <is>
-          <t>어둠의 족쇄</t>
+          <t>검은 부식</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="G40" t="inlineStr">
         <is>
-          <t>검은 부식</t>
+          <t>검은 압박</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="G41" t="inlineStr">
         <is>
-          <t>검은 압박</t>
+          <t>암흑</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="G42" t="inlineStr">
         <is>
-          <t>암흑</t>
+          <t>깊은 암흑</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="G43" t="inlineStr">
         <is>
-          <t>깊은 암흑</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: use vfx graph fireball for flame skills
</commit_message>
<xml_diff>
--- a/Project 2048/Docs/Project2048_Balancing_Template.xlsx
+++ b/Project 2048/Docs/Project2048_Balancing_Template.xlsx
@@ -9462,7 +9462,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>출혈 베기</t>
+          <t>화염구</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -10287,7 +10287,7 @@
       </c>
       <c r="Q16" s="79" t="inlineStr">
         <is>
-          <t>출혈 베기 기술을 배웁니다.</t>
+          <t>화염구 기술을 배웁니다.</t>
         </is>
       </c>
     </row>
@@ -10973,10 +10973,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing ns1:id="rId1"/>
+  <drawing r:id="rId1"/>
   <tableParts count="2">
-    <tablePart ns1:id="rId2"/>
-    <tablePart ns1:id="rId3"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: stabilize combat skill polish
</commit_message>
<xml_diff>
--- a/Project 2048/Docs/Project2048_Balancing_Template.xlsx
+++ b/Project 2048/Docs/Project2048_Balancing_Template.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
   <si>
     <t>Project 2048 밸런싱 대시보드</t>
   </si>
@@ -611,7 +611,7 @@
     <t>OverburnAttack</t>
   </si>
   <si>
-    <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다.</t>
+    <t>불꽃을 과열시켜 적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 불태우고, 추가 소모한 코스트 10당 위력 +10을 적용한다.</t>
   </si>
   <si>
     <t>poison-coat</t>
@@ -641,13 +641,16 @@
     <t>현재 보호막 수치로 계산하여 적에게 위력 60 피해를 준다. 보호막은 소모하지 않는다.</t>
   </si>
   <si>
-    <t>bleeding-cut</t>
+    <t>fireball</t>
   </si>
   <si>
     <t>화염구</t>
   </si>
   <si>
-    <t>적에게 위력 50 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 화염구를 발사한다.</t>
+    <t>BleedAttack</t>
+  </si>
+  <si>
+    <t>화염구를 발사해 적에게 위력 50 피해를 주고, 2턴 동안 턴 종료 시 20의 화상 피해를 준다.</t>
   </si>
   <si>
     <t>execute</t>
@@ -698,16 +701,16 @@
     <t>적에게 위력 90 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 1 감소한다.</t>
   </si>
   <si>
-    <t>blood-fang</t>
-  </si>
-  <si>
-    <t>불사르기</t>
+    <t>burn-out</t>
+  </si>
+  <si>
+    <t>화염 소모</t>
   </si>
   <si>
     <t>SacrificeAttack</t>
   </si>
   <si>
-    <t>최대 체력의 10%를 불태워 화염구를 발사하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
+    <t>자신의 최대 체력 10%를 불태워 거센 화염구를 발사하고 적에게 위력 100 피해를 준다. 이 비용으로 체력은 1 아래로 내려가지 않는다.</t>
   </si>
   <si>
     <t>body-press</t>
@@ -764,16 +767,19 @@
     <t>적에게 위력 60 피해를 준다. 실제 체력 피해의 50%만큼 체력을 회복한다.</t>
   </si>
   <si>
-    <t>open-wound</t>
-  </si>
-  <si>
-    <t>폭렬</t>
+    <t>burst-fireball</t>
+  </si>
+  <si>
+    <t>폭발 화염구</t>
+  </si>
+  <si>
+    <t>OpenWoundAttack</t>
   </si>
   <si>
     <t>70</t>
   </si>
   <si>
-    <t>적에게 위력 70 피해를 준다. 사용 후 남은 코스트를 모두 추가 소모하고, 추가 소모한 코스트 1당 위력 +10을 적용한다. 폭발하는 화염구를 발사하고, 적중 시 적 위치에 폭발 이펙트를 일으킨다.</t>
+    <t>폭발하는 화염구를 발사해 적에게 위력 70 피해를 준다. 대상이 독이나 화상 상태라면 위력 +50으로 공격하고, 해당 지속 피해 시간을 1턴 연장한다.</t>
   </si>
   <si>
     <t>shield-burst</t>
@@ -812,7 +818,7 @@
     <t>무리한 강타</t>
   </si>
   <si>
-    <t>적에게 위력 110 피해를 준다. 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
+    <t>몸을 사리지 않고 불꽃을 두른 강타로 적에게 위력 110 피해를 준다. 반동으로 다음 플레이어 턴의 보드 이동 횟수가 2 감소한다.</t>
   </si>
   <si>
     <t>crack-brand</t>
@@ -1178,9 +1184,6 @@
     <t>FearThenDarkness</t>
   </si>
   <si>
-    <t>출혈 베기</t>
-  </si>
-  <si>
     <t>Assets/Data/Enemies/01.asset</t>
   </si>
   <si>
@@ -1226,12 +1229,6 @@
     <t>물결치는 역병</t>
   </si>
   <si>
-    <t>피의 이빨</t>
-  </si>
-  <si>
-    <t>상처 벌리기</t>
-  </si>
-  <si>
     <t>Assets/Data/Enemies/06.asset</t>
   </si>
   <si>
@@ -1451,7 +1448,7 @@
     <t>생명 흡수 기술을 배웁니다.</t>
   </si>
   <si>
-    <t>learn-bleeding-cut</t>
+    <t>learn-fireball</t>
   </si>
   <si>
     <t>화염구 기술을 배웁니다.</t>
@@ -1463,10 +1460,10 @@
     <t>독 묻히기 기술을 배웁니다.</t>
   </si>
   <si>
-    <t>learn-open-wound</t>
-  </si>
-  <si>
-    <t>폭렬 기술을 배웁니다.</t>
+    <t>learn-burst-fireball</t>
+  </si>
+  <si>
+    <t>폭발 화염구 기술을 배웁니다.</t>
   </si>
   <si>
     <t>learn-execute</t>
@@ -1523,6 +1520,18 @@
     <t>빠른 승리</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>열1</t>
+  </si>
+  <si>
     <t>표준 승리</t>
   </si>
   <si>
@@ -1671,18 +1680,6 @@
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>열1</t>
   </si>
 </sst>
 </file>
@@ -5085,7 +5082,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -5372,7 +5369,7 @@
         <v>181</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>183</v>
@@ -5401,24 +5398,24 @@
         <v>250</v>
       </c>
       <c r="M9" s="24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N9" s="25" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="28.5">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C10" t="s">
         <v>181</v>
       </c>
       <c r="D10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E10" t="s">
         <v>183</v>
@@ -5447,30 +5444,30 @@
         <v>400</v>
       </c>
       <c r="M10" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="N10" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="28.5">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11" t="s">
         <v>181</v>
       </c>
       <c r="D11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E11" t="s">
         <v>183</v>
       </c>
       <c r="F11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G11">
         <v>6</v>
@@ -5493,18 +5490,18 @@
         <v>0</v>
       </c>
       <c r="M11" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N11" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C12" t="s">
         <v>181</v>
@@ -5516,7 +5513,7 @@
         <v>183</v>
       </c>
       <c r="F12" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G12">
         <v>6</v>
@@ -5539,24 +5536,24 @@
         <v>300</v>
       </c>
       <c r="M12" s="26" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="N12" s="26" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C13" t="s">
         <v>181</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E13" t="s">
         <v>183</v>
@@ -5585,24 +5582,24 @@
         <v>450</v>
       </c>
       <c r="M13" s="26" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N13" s="26" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C14" t="s">
         <v>181</v>
       </c>
       <c r="D14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E14" t="s">
         <v>183</v>
@@ -5631,27 +5628,27 @@
         <v>428.57142857142856</v>
       </c>
       <c r="M14" s="26" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N14" s="26" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C15" t="s">
         <v>181</v>
       </c>
       <c r="D15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F15" t="s">
         <v>184</v>
@@ -5677,30 +5674,30 @@
         <v>0</v>
       </c>
       <c r="M15" s="26" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N15" s="26" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C16" t="s">
         <v>181</v>
       </c>
       <c r="D16" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E16" t="s">
         <v>183</v>
       </c>
       <c r="F16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G16">
         <v>7</v>
@@ -5723,24 +5720,24 @@
         <v>214.28571428571428</v>
       </c>
       <c r="M16" s="26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="N16" s="26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C17" t="s">
         <v>181</v>
       </c>
       <c r="D17" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E17" t="s">
         <v>183</v>
@@ -5769,24 +5766,24 @@
         <v>214.28571428571428</v>
       </c>
       <c r="M17" s="26" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="N17" s="26" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:14">
       <c r="A18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B18" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C18" t="s">
         <v>181</v>
       </c>
       <c r="D18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E18" t="s">
         <v>183</v>
@@ -5815,24 +5812,24 @@
         <v>257.14285714285717</v>
       </c>
       <c r="M18" s="26" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="N18" s="26" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="42.75">
       <c r="A19" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B19" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C19" t="s">
         <v>181</v>
       </c>
       <c r="D19" t="s">
-        <v>188</v>
+        <v>243</v>
       </c>
       <c r="E19" t="s">
         <v>183</v>
@@ -5847,7 +5844,7 @@
         <v>70</v>
       </c>
       <c r="I19" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="J19" s="26">
         <f>IF(OR($C19&lt;&gt;"Attack",$I19&lt;=0),0,CEILING(($I19/10)*(IF($E19="ShieldHp",Inputs!$B$33,IF($E19="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
@@ -5861,24 +5858,24 @@
         <v>300</v>
       </c>
       <c r="M19" s="26" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N19" s="26" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B20" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C20" t="s">
         <v>181</v>
       </c>
       <c r="D20" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E20" t="s">
         <v>197</v>
@@ -5907,30 +5904,30 @@
         <v>42.857142857142854</v>
       </c>
       <c r="M20" s="26" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="N20" s="26" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C21" t="s">
         <v>181</v>
       </c>
       <c r="D21" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E21" t="s">
         <v>183</v>
       </c>
       <c r="F21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G21">
         <v>8</v>
@@ -5953,18 +5950,18 @@
         <v>450</v>
       </c>
       <c r="M21" s="26" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="N21" s="26" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B22" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C22" t="s">
         <v>181</v>
@@ -5999,24 +5996,24 @@
         <v>300</v>
       </c>
       <c r="M22" s="26" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N22" s="26" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B23" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C23" t="s">
         <v>181</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E23" t="s">
         <v>183</v>
@@ -6045,24 +6042,24 @@
         <v>412.5</v>
       </c>
       <c r="M23" s="26" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="N23" s="26" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="28.5">
       <c r="A24" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B24" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C24" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D24" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E24" t="s">
         <v>183</v>
@@ -6091,24 +6088,24 @@
         <v>0</v>
       </c>
       <c r="M24" s="26" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="N24" s="26" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B25" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C25" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D25" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E25" t="s">
         <v>183</v>
@@ -6137,24 +6134,24 @@
         <v>0</v>
       </c>
       <c r="M25" s="26" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="N25" s="26" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B26" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C26" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D26" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E26" t="s">
         <v>183</v>
@@ -6183,30 +6180,30 @@
         <v>0</v>
       </c>
       <c r="M26" s="26" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="N26" s="26" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="28.5">
       <c r="A27" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B27" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C27" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D27" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E27" t="s">
         <v>183</v>
       </c>
       <c r="F27" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G27">
         <v>5</v>
@@ -6229,24 +6226,24 @@
         <v>0</v>
       </c>
       <c r="M27" s="26" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="N27" s="26" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="28.5">
       <c r="A28" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B28" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C28" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D28" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E28" t="s">
         <v>183</v>
@@ -6275,30 +6272,30 @@
         <v>0</v>
       </c>
       <c r="M28" s="26" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="N28" s="26" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="28.5">
       <c r="A29" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B29" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C29" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D29" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E29" t="s">
         <v>183</v>
       </c>
       <c r="F29" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G29">
         <v>4</v>
@@ -6321,30 +6318,30 @@
         <v>0</v>
       </c>
       <c r="M29" s="26" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="N29" s="26" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="30" spans="1:14">
       <c r="A30" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B30" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C30" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E30" t="s">
         <v>183</v>
       </c>
       <c r="F30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G30">
         <v>4</v>
@@ -6367,24 +6364,24 @@
         <v>0</v>
       </c>
       <c r="M30" s="26" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="N30" s="26" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="31" spans="1:14">
       <c r="A31" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C31" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D31" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E31" t="s">
         <v>183</v>
@@ -6413,24 +6410,24 @@
         <v>0</v>
       </c>
       <c r="M31" s="26" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="N31" s="26" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B32" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D32" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E32" t="s">
         <v>183</v>
@@ -6459,30 +6456,30 @@
         <v>0</v>
       </c>
       <c r="M32" s="26" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="N32" s="26" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="33" spans="1:14">
       <c r="A33" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B33" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C33" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E33" t="s">
         <v>183</v>
       </c>
       <c r="F33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G33">
         <v>5</v>
@@ -6505,24 +6502,24 @@
         <v>0</v>
       </c>
       <c r="M33" s="26" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="N33" s="26" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="34" spans="1:14">
       <c r="A34" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B34" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C34" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D34" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E34" t="s">
         <v>183</v>
@@ -6551,24 +6548,24 @@
         <v>0</v>
       </c>
       <c r="M34" s="26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N34" s="26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="35" spans="1:14">
       <c r="A35" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B35" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C35" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D35" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E35" t="s">
         <v>183</v>
@@ -6597,30 +6594,30 @@
         <v>0</v>
       </c>
       <c r="M35" s="26" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="N35" s="26" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="36" spans="1:14">
       <c r="A36" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B36" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C36" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D36" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E36" t="s">
         <v>183</v>
       </c>
       <c r="F36" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G36">
         <v>6</v>
@@ -6643,30 +6640,30 @@
         <v>0</v>
       </c>
       <c r="M36" s="26" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="N36" s="26" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B37" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C37" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D37" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E37" t="s">
         <v>183</v>
       </c>
       <c r="F37" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G37">
         <v>6</v>
@@ -6689,24 +6686,24 @@
         <v>0</v>
       </c>
       <c r="M37" s="26" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="N37" s="26" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B38" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C38" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D38" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E38" t="s">
         <v>183</v>
@@ -6735,24 +6732,24 @@
         <v>0</v>
       </c>
       <c r="M38" s="26" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="N38" s="26" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="28.5">
       <c r="A39" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B39" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C39" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E39" t="s">
         <v>183</v>
@@ -6781,30 +6778,30 @@
         <v>0</v>
       </c>
       <c r="M39" s="26" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="N39" s="26" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="40" spans="1:14">
       <c r="A40" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B40" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C40" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D40" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E40" t="s">
         <v>183</v>
       </c>
       <c r="F40" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G40">
         <v>6</v>
@@ -6827,30 +6824,30 @@
         <v>0</v>
       </c>
       <c r="M40" s="26" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="N40" s="26" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="41" spans="1:14">
       <c r="A41" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B41" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C41" t="s">
         <v>181</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E41" t="s">
         <v>183</v>
       </c>
       <c r="F41" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G41">
         <v>0</v>
@@ -6873,30 +6870,30 @@
         <v/>
       </c>
       <c r="M41" s="26" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="N41" s="26" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="28.5">
       <c r="A42" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B42" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C42" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D42" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="E42" t="s">
         <v>183</v>
       </c>
       <c r="F42" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G42">
         <v>0</v>
@@ -6919,30 +6916,30 @@
         <v/>
       </c>
       <c r="M42" s="26" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="N42" s="26" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" t="s">
+        <v>340</v>
+      </c>
+      <c r="B43" t="s">
+        <v>341</v>
+      </c>
+      <c r="C43" t="s">
+        <v>261</v>
+      </c>
+      <c r="D43" t="s">
         <v>338</v>
-      </c>
-      <c r="B43" t="s">
-        <v>339</v>
-      </c>
-      <c r="C43" t="s">
-        <v>259</v>
-      </c>
-      <c r="D43" t="s">
-        <v>336</v>
       </c>
       <c r="E43" t="s">
         <v>183</v>
       </c>
       <c r="F43" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G43">
         <v>0</v>
@@ -6965,30 +6962,30 @@
         <v/>
       </c>
       <c r="M43" s="26" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="N43" s="26" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="44" spans="1:14">
       <c r="A44" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B44" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C44" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D44" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E44" t="s">
         <v>183</v>
       </c>
       <c r="F44" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G44">
         <v>0</v>
@@ -7011,30 +7008,30 @@
         <v/>
       </c>
       <c r="M44" s="26" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="N44" s="26" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" t="s">
+        <v>347</v>
+      </c>
+      <c r="B45" t="s">
+        <v>348</v>
+      </c>
+      <c r="C45" t="s">
+        <v>261</v>
+      </c>
+      <c r="D45" t="s">
         <v>345</v>
-      </c>
-      <c r="B45" t="s">
-        <v>346</v>
-      </c>
-      <c r="C45" t="s">
-        <v>259</v>
-      </c>
-      <c r="D45" t="s">
-        <v>343</v>
       </c>
       <c r="E45" t="s">
         <v>183</v>
       </c>
       <c r="F45" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G45">
         <v>0</v>
@@ -7057,10 +7054,10 @@
         <v/>
       </c>
       <c r="M45" s="26" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="N45" s="26" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -7082,28 +7079,28 @@
     <tablePart r:id="rId1"/>
   </tableParts>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0300-000000000000}">
-          <x14:formula1>
-            <xm:f>Lists!$A$2:$A$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>C5:C45</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0300-000001000000}">
-          <x14:formula1>
-            <xm:f>Lists!$H$2:$H$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>F5:F45</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns4:dataValidations count="2">
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0300-000000000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$A$2:$A$5</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>C5:C45</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0300-000001000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$H$2:$H$5</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>F5:F45</ns5:sqref>
+        </ns4:dataValidation>
+      </ns4:dataValidations>
     </ext>
   </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AA16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -7127,12 +7124,12 @@
   <sheetData>
     <row r="1" spans="1:27" ht="25.5" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="19.5" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
@@ -7182,99 +7179,99 @@
         <v>8</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F4" s="20" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K4" s="20" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="L4" s="20" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="M4" s="20" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="N4" s="20" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="O4" s="20" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="P4" s="20" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="Q4" s="20" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="R4" s="20" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="S4" s="20" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="T4" s="20" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="U4" s="20" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="V4" s="20" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="W4" s="20" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="X4" s="20" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="Y4" s="20" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="Z4" s="20" t="s">
         <v>31</v>
       </c>
       <c r="AA4" s="20" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="2" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F5" s="12">
         <v>150</v>
@@ -7307,13 +7304,13 @@
         <v>180</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>378</v>
+        <v>200</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="S5" s="27">
         <f>IF($D5="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D5="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7348,24 +7345,24 @@
         <v>23.7</v>
       </c>
       <c r="AA5" s="26" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="6" spans="1:27">
       <c r="A6" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F6" s="12">
         <v>190</v>
@@ -7395,16 +7392,16 @@
         <v>3</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="S6" s="27">
         <f>IF($D6="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D6="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7439,24 +7436,24 @@
         <v>25.8</v>
       </c>
       <c r="AA6" s="26" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:27">
       <c r="A7" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F7" s="12">
         <v>140</v>
@@ -7489,13 +7486,13 @@
         <v>191</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="S7" s="27">
         <f>IF($D7="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D7="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7530,24 +7527,24 @@
         <v>19.8</v>
       </c>
       <c r="AA7" s="26" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="8" spans="1:27">
       <c r="A8" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F8" s="12">
         <v>180</v>
@@ -7577,16 +7574,16 @@
         <v>3</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="S8" s="27">
         <f>IF($D8="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D8="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7621,24 +7618,24 @@
         <v>25.1</v>
       </c>
       <c r="AA8" s="26" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" spans="1:27">
       <c r="A9" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F9" s="12">
         <v>150</v>
@@ -7671,13 +7668,13 @@
         <v>180</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>378</v>
+        <v>200</v>
       </c>
       <c r="S9" s="27">
         <f>IF($D9="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D9="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7712,24 +7709,24 @@
         <v>95.7</v>
       </c>
       <c r="AA9" s="26" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:27">
       <c r="A10" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F10" s="12">
         <v>210</v>
@@ -7759,16 +7756,16 @@
         <v>2</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>394</v>
+        <v>220</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>395</v>
+        <v>242</v>
       </c>
       <c r="S10" s="27">
         <f>IF($D10="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D10="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7803,24 +7800,24 @@
         <v>133.69999999999999</v>
       </c>
       <c r="AA10" s="26" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="11" spans="1:27">
       <c r="A11" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F11" s="12">
         <v>170</v>
@@ -7853,13 +7850,13 @@
         <v>191</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>395</v>
+        <v>242</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="S11" s="27">
         <f>IF($D11="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D11="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7894,24 +7891,24 @@
         <v>70.8</v>
       </c>
       <c r="AA11" s="26" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:27">
       <c r="A12" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F12" s="12">
         <v>220</v>
@@ -7944,13 +7941,13 @@
         <v>187</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q12" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="S12" s="27">
         <f>IF($D12="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D12="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -7985,24 +7982,24 @@
         <v>134</v>
       </c>
       <c r="AA12" s="26" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="13" spans="1:27">
       <c r="A13" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>402</v>
-      </c>
       <c r="E13" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F13" s="12">
         <v>180</v>
@@ -8032,16 +8029,16 @@
         <v>3</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="Q13" s="4" t="s">
         <v>195</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="S13" s="27">
         <f>IF($D13="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D13="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -8076,24 +8073,24 @@
         <v>27.1</v>
       </c>
       <c r="AA13" s="26" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" spans="1:27">
       <c r="A14" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F14" s="12">
         <v>240</v>
@@ -8123,16 +8120,16 @@
         <v>3</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Q14" s="4" t="s">
-        <v>395</v>
+        <v>242</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="S14" s="27">
         <f>IF($D14="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D14="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -8167,24 +8164,24 @@
         <v>47.9</v>
       </c>
       <c r="AA14" s="26" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:27">
       <c r="A15" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>407</v>
-      </c>
       <c r="C15" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F15" s="12">
         <v>200</v>
@@ -8214,16 +8211,16 @@
         <v>4</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="Q15" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="S15" s="27">
         <f>IF($D15="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D15="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -8258,24 +8255,24 @@
         <v>38.200000000000003</v>
       </c>
       <c r="AA15" s="26" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16" spans="1:27">
       <c r="A16" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>410</v>
-      </c>
       <c r="C16" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F16" s="12">
         <v>230</v>
@@ -8305,16 +8302,16 @@
         <v>3</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="R16" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="S16" s="27">
         <f>IF($D16="AttackHeavy",Inputs!$B$21/(Inputs!$B$21+Inputs!$B$22),IF($D16="DefenseHeavy",Inputs!$B$23/(Inputs!$B$23+Inputs!$B$24),Inputs!$B$19/(Inputs!$B$19+Inputs!$B$20)))</f>
@@ -8349,7 +8346,7 @@
         <v>47.6</v>
       </c>
       <c r="AA16" s="26" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -8371,40 +8368,40 @@
     <tablePart r:id="rId1"/>
   </tableParts>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0400-000000000000}">
-          <x14:formula1>
-            <xm:f>Lists!$D$2:$D$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>B5:B16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0400-000001000000}">
-          <x14:formula1>
-            <xm:f>Lists!$E$2:$E$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>C5:C16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0400-000002000000}">
-          <x14:formula1>
-            <xm:f>Lists!$B$2:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>D5:D16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0400-000003000000}">
-          <x14:formula1>
-            <xm:f>Lists!$C$2:$C$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>E5:E16</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns4:dataValidations count="4">
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0400-000000000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$D$2:$D$5</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>B5:B16</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0400-000001000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$E$2:$E$3</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>C5:C16</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0400-000002000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$B$2:$B$4</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>D5:D16</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0400-000003000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$C$2:$C$3</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>E5:E16</ns5:sqref>
+        </ns4:dataValidation>
+      </ns4:dataValidations>
     </ext>
   </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:Q24"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -8425,12 +8422,12 @@
   <sheetData>
     <row r="1" spans="1:17" ht="25.5" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1">
       <c r="A2" s="19" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
@@ -8463,7 +8460,7 @@
     </row>
     <row r="4" spans="1:17" ht="30">
       <c r="A4" s="20" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>8</v>
@@ -8472,34 +8469,34 @@
         <v>20</v>
       </c>
       <c r="D4" s="20" t="s">
+        <v>414</v>
+      </c>
+      <c r="E4" s="20" t="s">
         <v>415</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="F4" s="20" t="s">
         <v>416</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="G4" s="20" t="s">
         <v>417</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="H4" s="20" t="s">
         <v>418</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="I4" s="20" t="s">
         <v>419</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>420</v>
       </c>
       <c r="J4" s="20" t="s">
         <v>23</v>
       </c>
       <c r="K4" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="L4" s="20" t="s">
         <v>421</v>
       </c>
-      <c r="L4" s="20" t="s">
+      <c r="M4" s="20" t="s">
         <v>422</v>
-      </c>
-      <c r="M4" s="20" t="s">
-        <v>423</v>
       </c>
       <c r="N4" s="20" t="s">
         <v>17</v>
@@ -8511,7 +8508,7 @@
         <v>11</v>
       </c>
       <c r="Q4" s="20" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -8519,7 +8516,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C5" s="12">
         <v>6</v>
@@ -8531,10 +8528,10 @@
         <v>0</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H5" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B5,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8573,7 +8570,7 @@
         <v>OK</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -8581,7 +8578,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C6" s="12">
         <v>6</v>
@@ -8593,10 +8590,10 @@
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H6" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B6,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8635,7 +8632,7 @@
         <v>OK</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -8643,7 +8640,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C7" s="12">
         <v>6</v>
@@ -8655,10 +8652,10 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H7" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B7,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8697,7 +8694,7 @@
         <v>OK</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -8705,7 +8702,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C8" s="12">
         <v>6</v>
@@ -8717,10 +8714,10 @@
         <v>0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H8" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B8,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8759,7 +8756,7 @@
         <v>OK</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -8767,7 +8764,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C9" s="12">
         <v>8</v>
@@ -8779,10 +8776,10 @@
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H9" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B9,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8821,7 +8818,7 @@
         <v>OK</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -8829,7 +8826,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C10" s="12">
         <v>8</v>
@@ -8841,10 +8838,10 @@
         <v>0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H10" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B10,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8883,7 +8880,7 @@
         <v>주의</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -8891,7 +8888,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C11" s="12">
         <v>8</v>
@@ -8903,10 +8900,10 @@
         <v>0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H11" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B11,Enemies!$A$5:$A$16,0)),"")</f>
@@ -8945,7 +8942,7 @@
         <v>OK</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -8953,7 +8950,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C12" s="12">
         <v>8</v>
@@ -8965,10 +8962,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H12" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B12,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9007,7 +9004,7 @@
         <v>주의</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -9015,7 +9012,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C13" s="12">
         <v>8</v>
@@ -9027,10 +9024,10 @@
         <v>0</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H13" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B13,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9069,7 +9066,7 @@
         <v>OK</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -9077,7 +9074,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C14" s="12">
         <v>8</v>
@@ -9089,10 +9086,10 @@
         <v>0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H14" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B14,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9131,7 +9128,7 @@
         <v>OK</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -9139,7 +9136,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C15" s="12">
         <v>8</v>
@@ -9151,10 +9148,10 @@
         <v>0</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H15" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B15,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9193,7 +9190,7 @@
         <v>OK</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -9201,7 +9198,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C16" s="12">
         <v>8</v>
@@ -9213,10 +9210,10 @@
         <v>0</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H16" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B16,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9255,7 +9252,7 @@
         <v>OK</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -9263,7 +9260,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C17" s="12">
         <v>8</v>
@@ -9275,10 +9272,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H17" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B17,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9317,7 +9314,7 @@
         <v>OK</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -9325,7 +9322,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C18" s="12">
         <v>8</v>
@@ -9337,10 +9334,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H18" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B18,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9379,7 +9376,7 @@
         <v>OK</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -9387,7 +9384,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C19" s="12">
         <v>8</v>
@@ -9399,10 +9396,10 @@
         <v>0</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H19" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B19,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9441,7 +9438,7 @@
         <v>OK</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -9449,7 +9446,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C20" s="12">
         <v>8</v>
@@ -9461,10 +9458,10 @@
         <v>0</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H20" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B20,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9503,7 +9500,7 @@
         <v>OK</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -9511,7 +9508,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C21" s="12">
         <v>8</v>
@@ -9523,10 +9520,10 @@
         <v>0</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H21" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B21,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9565,7 +9562,7 @@
         <v>OK</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -9573,7 +9570,7 @@
         <v>18</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C22" s="12">
         <v>8</v>
@@ -9585,10 +9582,10 @@
         <v>0</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H22" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B22,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9627,7 +9624,7 @@
         <v>주의</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -9635,7 +9632,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C23" s="12">
         <v>8</v>
@@ -9647,10 +9644,10 @@
         <v>0</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H23" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B23,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9689,7 +9686,7 @@
         <v>OK</v>
       </c>
       <c r="Q23" s="2" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -9697,7 +9694,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C24" s="12">
         <v>8</v>
@@ -9709,10 +9706,10 @@
         <v>0</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H24" s="4">
         <f>IFERROR(INDEX(Enemies!$F$5:$F$16,MATCH($B24,Enemies!$A$5:$A$16,0)),"")</f>
@@ -9751,7 +9748,7 @@
         <v>주의</v>
       </c>
       <c r="Q24" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -9766,28 +9763,28 @@
     <tablePart r:id="rId1"/>
   </tableParts>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0500-000000000000}">
-          <x14:formula1>
-            <xm:f>Lists!$F$2:$F$13</xm:f>
-          </x14:formula1>
-          <xm:sqref>B5:B24</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0500-000001000000}">
-          <x14:formula1>
-            <xm:f>Lists!$G$2:$G$43</xm:f>
-          </x14:formula1>
-          <xm:sqref>F5:G24</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns4:dataValidations count="2">
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0500-000000000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$F$2:$F$13</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>B5:B24</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0500-000001000000}">
+          <ns4:formula1>
+            <ns5:f>Lists!$G$2:$G$43</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>F5:G24</ns5:sqref>
+        </ns4:dataValidation>
+      </ns4:dataValidations>
     </ext>
   </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -9803,12 +9800,12 @@
   <sheetData>
     <row r="1" spans="1:17" ht="25.5" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -9817,66 +9814,66 @@
     </row>
     <row r="4" spans="1:17" ht="45">
       <c r="A4" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>426</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="C4" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="D4" s="20" t="s">
         <v>428</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="E4" s="20" t="s">
         <v>429</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="F4" s="20" t="s">
         <v>430</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="G4" s="20" t="s">
         <v>431</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="H4" s="20" t="s">
         <v>432</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="I4" s="20" t="s">
         <v>433</v>
       </c>
-      <c r="I4" s="20" t="s">
+      <c r="J4" s="20" t="s">
         <v>434</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="K4" s="20" t="s">
         <v>435</v>
       </c>
-      <c r="K4" s="20" t="s">
+      <c r="L4" s="20" t="s">
         <v>436</v>
       </c>
-      <c r="L4" s="20" t="s">
+      <c r="M4" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="M4" s="20" t="s">
+      <c r="N4" s="20" t="s">
         <v>438</v>
       </c>
-      <c r="N4" s="20" t="s">
+      <c r="O4" s="20" t="s">
         <v>439</v>
       </c>
-      <c r="O4" s="20" t="s">
+      <c r="P4" s="20" t="s">
         <v>440</v>
       </c>
-      <c r="P4" s="20" t="s">
+      <c r="Q4" s="20" t="s">
         <v>441</v>
-      </c>
-      <c r="Q4" s="20" t="s">
-        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="16" t="s">
         <v>444</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>445</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="5">
@@ -9912,21 +9909,21 @@
         <v>0.1</v>
       </c>
       <c r="Q5" s="26" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="28" t="s">
+        <v>446</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>448</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>449</v>
-      </c>
       <c r="D6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E6" s="8">
         <v>0.3</v>
@@ -9961,21 +9958,21 @@
         <v>0.1</v>
       </c>
       <c r="Q6" s="26" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>448</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>449</v>
-      </c>
       <c r="D7" s="8" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E7" s="8">
         <v>0.3</v>
@@ -10010,21 +10007,21 @@
         <v>0.1</v>
       </c>
       <c r="Q7" s="26" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C8" t="s">
         <v>448</v>
       </c>
-      <c r="C8" t="s">
-        <v>449</v>
-      </c>
       <c r="D8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E8">
         <v>0.3</v>
@@ -10059,21 +10056,21 @@
         <v>0.1</v>
       </c>
       <c r="Q8" s="26" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="7" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>449</v>
-      </c>
       <c r="D9" s="7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E9" s="7">
         <v>0.3</v>
@@ -10108,21 +10105,21 @@
         <v>0.1</v>
       </c>
       <c r="Q9" s="26" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B10" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>449</v>
-      </c>
       <c r="D10" s="12" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E10" s="12">
         <v>0.3</v>
@@ -10157,21 +10154,21 @@
         <v>0.1</v>
       </c>
       <c r="Q10" s="26" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="25" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B11" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>449</v>
-      </c>
       <c r="D11" s="12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E11" s="12">
         <v>0.3</v>
@@ -10206,21 +10203,21 @@
         <v>0.1</v>
       </c>
       <c r="Q11" s="26" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>449</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E12" s="12">
         <v>0.3</v>
@@ -10255,21 +10252,21 @@
         <v>0.1</v>
       </c>
       <c r="Q12" s="26" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B13" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>449</v>
-      </c>
       <c r="D13" s="12" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E13" s="12">
         <v>0.3</v>
@@ -10304,21 +10301,21 @@
         <v>0.1</v>
       </c>
       <c r="Q13" s="26" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B14" t="s">
+        <v>447</v>
+      </c>
+      <c r="C14" t="s">
         <v>448</v>
       </c>
-      <c r="C14" t="s">
-        <v>449</v>
-      </c>
       <c r="D14" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E14">
         <v>0.3</v>
@@ -10353,21 +10350,21 @@
         <v>0.1</v>
       </c>
       <c r="Q14" s="26" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B15" t="s">
+        <v>447</v>
+      </c>
+      <c r="C15" t="s">
         <v>448</v>
       </c>
-      <c r="C15" t="s">
-        <v>449</v>
-      </c>
       <c r="D15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E15">
         <v>0.3</v>
@@ -10402,18 +10399,18 @@
         <v>0.1</v>
       </c>
       <c r="Q15" s="26" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B16" t="s">
+        <v>447</v>
+      </c>
+      <c r="C16" t="s">
         <v>448</v>
-      </c>
-      <c r="C16" t="s">
-        <v>449</v>
       </c>
       <c r="D16" t="s">
         <v>200</v>
@@ -10451,18 +10448,18 @@
         <v>0.1</v>
       </c>
       <c r="Q16" s="26" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C17" t="s">
         <v>448</v>
-      </c>
-      <c r="C17" t="s">
-        <v>449</v>
       </c>
       <c r="D17" t="s">
         <v>191</v>
@@ -10500,21 +10497,21 @@
         <v>0.1</v>
       </c>
       <c r="Q17" s="26" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C18" t="s">
         <v>448</v>
       </c>
-      <c r="C18" t="s">
-        <v>449</v>
-      </c>
       <c r="D18" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E18">
         <v>0.3</v>
@@ -10549,21 +10546,21 @@
         <v>0.1</v>
       </c>
       <c r="Q18" s="26" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="19" spans="1:17">
       <c r="A19" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B19" t="s">
+        <v>447</v>
+      </c>
+      <c r="C19" t="s">
         <v>448</v>
       </c>
-      <c r="C19" t="s">
-        <v>449</v>
-      </c>
       <c r="D19" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E19">
         <v>0.3</v>
@@ -10598,18 +10595,18 @@
         <v>0.1</v>
       </c>
       <c r="Q19" s="26" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="20" spans="1:17">
       <c r="A20" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B20" t="s">
+        <v>447</v>
+      </c>
+      <c r="C20" t="s">
         <v>448</v>
-      </c>
-      <c r="C20" t="s">
-        <v>449</v>
       </c>
       <c r="D20" t="s">
         <v>187</v>
@@ -10647,21 +10644,21 @@
         <v>0.1</v>
       </c>
       <c r="Q20" s="26" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C21" t="s">
         <v>448</v>
       </c>
-      <c r="C21" t="s">
-        <v>449</v>
-      </c>
       <c r="D21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E21">
         <v>0.3</v>
@@ -10696,21 +10693,21 @@
         <v>0.1</v>
       </c>
       <c r="Q21" s="26" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B22" t="s">
+        <v>447</v>
+      </c>
+      <c r="C22" t="s">
         <v>448</v>
       </c>
-      <c r="C22" t="s">
-        <v>449</v>
-      </c>
       <c r="D22" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E22">
         <v>0.3</v>
@@ -10745,21 +10742,21 @@
         <v>0.1</v>
       </c>
       <c r="Q22" s="26" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B23" t="s">
+        <v>447</v>
+      </c>
+      <c r="C23" t="s">
         <v>448</v>
       </c>
-      <c r="C23" t="s">
-        <v>449</v>
-      </c>
       <c r="D23" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E23">
         <v>0.3</v>
@@ -10794,21 +10791,21 @@
         <v>0.1</v>
       </c>
       <c r="Q23" s="26" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B24" t="s">
+        <v>447</v>
+      </c>
+      <c r="C24" t="s">
         <v>448</v>
       </c>
-      <c r="C24" t="s">
-        <v>449</v>
-      </c>
       <c r="D24" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E24">
         <v>0.3</v>
@@ -10843,21 +10840,21 @@
         <v>0.1</v>
       </c>
       <c r="Q24" s="26" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B25" t="s">
+        <v>447</v>
+      </c>
+      <c r="C25" t="s">
         <v>448</v>
       </c>
-      <c r="C25" t="s">
-        <v>449</v>
-      </c>
       <c r="D25" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E25">
         <v>0.3</v>
@@ -10892,7 +10889,7 @@
         <v>0.1</v>
       </c>
       <c r="Q25" s="26" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -10907,19 +10904,19 @@
     </row>
     <row r="28" spans="1:17" ht="30">
       <c r="A28" s="20" t="s">
+        <v>488</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>489</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="C28" s="20" t="s">
+        <v>414</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="E28" s="20" t="s">
         <v>490</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>415</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>416</v>
-      </c>
-      <c r="E28" s="20" t="s">
-        <v>491</v>
       </c>
       <c r="F28" s="20" t="s">
         <v>14</v>
@@ -10930,22 +10927,22 @@
     </row>
     <row r="29" spans="1:17" ht="15">
       <c r="A29" t="s">
+        <v>491</v>
+      </c>
+      <c r="B29" t="s">
         <v>492</v>
       </c>
-      <c r="B29" t="s">
-        <v>543</v>
-      </c>
       <c r="C29" t="s">
-        <v>544</v>
+        <v>493</v>
       </c>
       <c r="D29" t="s">
         <v>85</v>
       </c>
       <c r="E29" t="s">
-        <v>545</v>
+        <v>494</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>546</v>
+        <v>495</v>
       </c>
       <c r="H29" s="26"/>
       <c r="I29" s="26"/>
@@ -10953,7 +10950,7 @@
     </row>
     <row r="30" spans="1:17">
       <c r="A30" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="B30">
         <v>1</v>
@@ -10977,7 +10974,7 @@
     </row>
     <row r="31" spans="1:17">
       <c r="A31" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="B31">
         <v>2</v>
@@ -11001,7 +10998,7 @@
     </row>
     <row r="32" spans="1:17">
       <c r="A32" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B32">
         <v>2</v>
@@ -11035,7 +11032,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -11049,14 +11046,14 @@
   <sheetData>
     <row r="1" spans="1:8" ht="25.5" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="G1" s="8"/>
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -11071,41 +11068,41 @@
     </row>
     <row r="4" spans="1:8" ht="15">
       <c r="A4" s="20" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" ht="34.5" customHeight="1">
       <c r="A5" s="17" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="8"/>
@@ -11113,19 +11110,19 @@
     </row>
     <row r="6" spans="1:8" ht="34.5" customHeight="1">
       <c r="A6" s="17" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="C6" s="17" t="s">
+        <v>514</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>515</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>511</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>512</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>508</v>
       </c>
       <c r="F6" s="17"/>
       <c r="G6" s="8"/>
@@ -11133,41 +11130,41 @@
     </row>
     <row r="7" spans="1:8" ht="34.5" customHeight="1">
       <c r="A7" s="17" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
     </row>
     <row r="8" spans="1:8" ht="34.5" customHeight="1">
       <c r="A8" s="17" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="F8" s="17"/>
       <c r="G8" s="8"/>
@@ -11175,41 +11172,41 @@
     </row>
     <row r="9" spans="1:8" ht="34.5" customHeight="1">
       <c r="A9" s="17" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" ht="34.5" customHeight="1">
       <c r="A10" s="17" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B10" s="17" t="s">
+        <v>532</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>533</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>534</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>529</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>530</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>531</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>526</v>
       </c>
       <c r="F10" s="17"/>
       <c r="G10" s="8"/>
@@ -11235,7 +11232,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:I43"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -11247,31 +11244,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15">
       <c r="A1" s="20" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B1" s="20" t="s">
+        <v>354</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>355</v>
+      </c>
+      <c r="D1" s="20" t="s">
         <v>352</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="E1" s="20" t="s">
         <v>353</v>
       </c>
-      <c r="D1" s="20" t="s">
-        <v>350</v>
-      </c>
-      <c r="E1" s="20" t="s">
-        <v>351</v>
-      </c>
       <c r="F1" s="20" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="H1" s="20" t="s">
         <v>170</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -11279,19 +11276,19 @@
         <v>181</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>374</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>180</v>
@@ -11300,84 +11297,84 @@
         <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>390</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>187</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I3" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>191</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="I4" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>195</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="I5" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -11387,14 +11384,14 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>378</v>
+        <v>200</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -11404,10 +11401,10 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H7" s="2"/>
     </row>
@@ -11418,10 +11415,10 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H8" s="2"/>
     </row>
@@ -11432,10 +11429,10 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H9" s="2"/>
     </row>
@@ -11446,10 +11443,10 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H10" s="2"/>
     </row>
@@ -11460,10 +11457,10 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>394</v>
+        <v>220</v>
       </c>
       <c r="H11" s="2"/>
     </row>
@@ -11474,10 +11471,10 @@
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H12" s="2"/>
     </row>
@@ -11488,10 +11485,10 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H13" s="2"/>
     </row>
@@ -11503,7 +11500,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H14" s="2"/>
     </row>
@@ -11515,7 +11512,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H15" s="2"/>
     </row>
@@ -11527,7 +11524,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
-        <v>395</v>
+        <v>242</v>
       </c>
       <c r="H16" s="2"/>
     </row>
@@ -11539,7 +11536,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H17" s="2"/>
     </row>
@@ -11551,7 +11548,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="H18" s="2"/>
     </row>
@@ -11563,7 +11560,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H19" s="2"/>
     </row>
@@ -11575,7 +11572,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H20" s="2"/>
     </row>
@@ -11587,7 +11584,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="H21" s="2"/>
     </row>
@@ -11599,7 +11596,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="H22" s="2"/>
     </row>
@@ -11611,7 +11608,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -11623,7 +11620,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H24" s="2"/>
     </row>
@@ -11635,7 +11632,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="H25" s="2"/>
     </row>
@@ -11647,7 +11644,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="H26" s="2"/>
     </row>
@@ -11659,7 +11656,7 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H27" s="2"/>
     </row>
@@ -11671,7 +11668,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="H28" s="2"/>
     </row>
@@ -11683,7 +11680,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H29" s="2"/>
     </row>
@@ -11695,73 +11692,73 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:8">
       <c r="G31" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="G32" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="33" spans="7:7">
       <c r="G33" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="34" spans="7:7">
       <c r="G34" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="35" spans="7:7">
       <c r="G35" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="36" spans="7:7">
       <c r="G36" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="37" spans="7:7">
       <c r="G37" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="38" spans="7:7">
       <c r="G38" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="39" spans="7:7">
       <c r="G39" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="40" spans="7:7">
       <c r="G40" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="41" spans="7:7">
       <c r="G41" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="42" spans="7:7">
       <c r="G42" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="43" spans="7:7">
       <c r="G43" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: tune starter skill balance
</commit_message>
<xml_diff>
--- a/Project 2048/Docs/Project2048_Balancing_Template.xlsx
+++ b/Project 2048/Docs/Project2048_Balancing_Template.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="552">
   <si>
     <t>Project 2048 밸런싱 대시보드</t>
   </si>
@@ -1680,6 +1680,24 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>?? ? ?? ???? 15 ????.</t>
+  </si>
+  <si>
+    <t>??? 20? ???.</t>
+  </si>
+  <si>
+    <t>??? 40? ???.</t>
+  </si>
+  <si>
+    <t>다음 턴 시작 코스트가 15 증가한다.</t>
+  </si>
+  <si>
+    <t>보호막 20을 얻는다.</t>
+  </si>
+  <si>
+    <t>보호막 40을 얻는다.</t>
   </si>
 </sst>
 </file>
@@ -5082,7 +5100,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -6318,10 +6336,10 @@
         <v>0</v>
       </c>
       <c r="M29" s="26" t="s">
-        <v>286</v>
+        <v>549</v>
       </c>
       <c r="N29" s="26" t="s">
-        <v>286</v>
+        <v>549</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -6439,27 +6457,27 @@
         <v>4</v>
       </c>
       <c r="H32">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="I32">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J32" s="26">
         <f>IF(OR($C32&lt;&gt;"Attack",$I32&lt;=0),0,CEILING(($I32/10)*(IF($E32="ShieldHp",Inputs!$B$33,IF($E32="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v>0</v>
       </c>
       <c r="K32">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="L32" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M32" s="26" t="s">
-        <v>299</v>
+        <v>550</v>
       </c>
       <c r="N32" s="26" t="s">
-        <v>299</v>
+        <v>550</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -6623,27 +6641,27 @@
         <v>6</v>
       </c>
       <c r="H36">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="J36" s="26">
         <f>IF(OR($C36&lt;&gt;"Attack",$I36&lt;=0),0,CEILING(($I36/10)*(IF($E36="ShieldHp",Inputs!$B$33,IF($E36="DefensePower",Inputs!$B$28,Inputs!$B$5))/MAX(1,Inputs!$B$32))*Inputs!$B$34,1))</f>
         <v>0</v>
       </c>
       <c r="K36">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="L36" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M36" s="26" t="s">
-        <v>315</v>
+        <v>551</v>
       </c>
       <c r="N36" s="26" t="s">
-        <v>315</v>
+        <v>551</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -7076,7 +7094,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart ns3:id="rId1"/>
   </tableParts>
   <extLst>
     <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>